<commit_message>
Clarify AI adoption diagnostic value
</commit_message>
<xml_diff>
--- a/products/AI_Tool_Selection_Checklist_v0.1.xlsx
+++ b/products/AI_Tool_Selection_Checklist_v0.1.xlsx
@@ -2,12 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start" sheetId="1" r:id="R745eb832436b4146"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tool Matrix" sheetId="2" r:id="Rd8055f5e16374535"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Use Case Scores" sheetId="3" r:id="R2ad28655030040fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Automation Recipes" sheetId="4" r:id="Re532c57516ac4000"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt Pack" sheetId="5" r:id="Rd2ef270f6cc449f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Rd0778fa80b9843e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start" sheetId="1" r:id="R4cc2e84383bd4c71"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Inventory" sheetId="2" r:id="R6f54f84a0f714638"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROI Calculator" sheetId="3" r:id="R51873790ba8a429b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Summary" sheetId="4" r:id="R76a514304d0c47a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tool Matrix" sheetId="5" r:id="Rc4e00a7ec5644a96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Use Case Scores" sheetId="6" r:id="R40826377ec9e463a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Automation Recipes" sheetId="7" r:id="R49bb289fc74f44b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt Pack" sheetId="8" r:id="R25a637bba2d04737"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="9" r:id="Rda424072508f41b3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18,9 +21,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="2">
-    <x:numFmt numFmtId="200" formatCode="¥#,##0"/>
-    <x:numFmt numFmtId="201" formatCode="0"/>
+  <x:numFmts count="4">
+    <x:numFmt numFmtId="200" formatCode="0.0"/>
+    <x:numFmt numFmtId="201" formatCode="¥#,##0"/>
+    <x:numFmt numFmtId="202" formatCode="0%"/>
+    <x:numFmt numFmtId="203" formatCode="0"/>
   </x:numFmts>
   <x:fonts count="4">
     <x:font>
@@ -69,7 +74,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="16">
+  <x:cellXfs count="18">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -104,6 +109,12 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="201" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -273,7 +284,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="5" t="str">
-        <x:v>小規模事業者・副業ワーカーが、AIツールを雰囲気ではなく用途・費用・運用しやすさで選ぶための実務テンプレートです。</x:v>
+        <x:v>小規模事業者・副業ワーカーが、AIツールを買う前に「どの作業をAI化すべきか」「何時間浮くか」「どの構成で始めるか」を決めるための診断キットです。</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="21" customHeight="1">
@@ -281,31 +292,31 @@
         <x:v>使い方</x:v>
       </x:c>
       <x:c r="B5" s="8" t="str">
-        <x:v>Tool Matrixに候補ツールを入力</x:v>
+        <x:v>Task Inventoryに毎週の手作業を10個書き出す</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="21" customHeight="1">
       <x:c r="A6" s="7" t="str"/>
       <x:c r="B6" s="8" t="str">
-        <x:v>Use Case Scoresで用途別に1から5点で採点</x:v>
+        <x:v>ROI Calculatorで削減時間と月額コストを比較する</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="21" customHeight="1">
       <x:c r="A7" s="7" t="str"/>
       <x:c r="B7" s="8" t="str">
-        <x:v>合計点と月額コストを見て導入候補を絞る</x:v>
+        <x:v>Decision Summaryで最初に試すAI化候補を1つに絞る</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="21" customHeight="1">
       <x:c r="A8" s="7" t="str"/>
       <x:c r="B8" s="8" t="str">
-        <x:v>Automation Recipesから最初に試す業務を選ぶ</x:v>
+        <x:v>Tool Matrixで必要なツール構成だけを選ぶ</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="21" customHeight="1">
       <x:c r="A9" s="7" t="str"/>
       <x:c r="B9" s="8" t="str">
-        <x:v>Prompt Packをコピーして自社向けに調整</x:v>
+        <x:v>Prompt Packをコピーして自社向けに調整する</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="21" customHeight="1">
@@ -340,6 +351,700 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="24.899999618530273" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="5.519999980926514" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14.800000190734863" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="11.710000038146973" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="6.460000038146973" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="12.380000114440918" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="15.75" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="4.170000076293945" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="6.059999942779541" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="28.940000534057617" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="33" hidden="0" customHeight="1">
+      <x:c r="A1" s="13" t="str">
+        <x:v>Task</x:v>
+      </x:c>
+      <x:c r="B1" s="13" t="str">
+        <x:v>Owner</x:v>
+      </x:c>
+      <x:c r="C1" s="13" t="str">
+        <x:v>Frequency / Week</x:v>
+      </x:c>
+      <x:c r="D1" s="13" t="str">
+        <x:v>Minutes / Run</x:v>
+      </x:c>
+      <x:c r="E1" s="13" t="str">
+        <x:v>Pain 1-5</x:v>
+      </x:c>
+      <x:c r="F1" s="13" t="str">
+        <x:v>Rule Clarity 1-5</x:v>
+      </x:c>
+      <x:c r="G1" s="13" t="str">
+        <x:v>Data Sensitivity 1-5</x:v>
+      </x:c>
+      <x:c r="H1" s="13" t="str">
+        <x:v>AI Fit</x:v>
+      </x:c>
+      <x:c r="I1" s="13" t="str">
+        <x:v>Priority</x:v>
+      </x:c>
+      <x:c r="J1" s="13" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="33" hidden="0" customHeight="1">
+      <x:c r="A2" s="9" t="str">
+        <x:v>問い合わせ返信の下書き</x:v>
+      </x:c>
+      <x:c r="B2" s="9" t="str">
+        <x:v>Owner</x:v>
+      </x:c>
+      <x:c r="C2" s="9" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D2" s="9" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E2" s="9" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F2" s="9" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G2" s="9" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H2" s="9" t="n">
+        <x:f>ROUND(((E2+F2)*2-G2)/2,1)</x:f>
+        <x:v>6.5</x:v>
+      </x:c>
+      <x:c r="I2" s="9" t="str">
+        <x:f>IF(H2&gt;=7,"Start",IF(H2&gt;=5,"Test","Skip"))</x:f>
+        <x:v>Test</x:v>
+      </x:c>
+      <x:c r="J2" s="9" t="str">
+        <x:v>送信前は人間確認</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="33" hidden="0" customHeight="1">
+      <x:c r="A3" s="9" t="str">
+        <x:v>SNS投稿案の作成</x:v>
+      </x:c>
+      <x:c r="B3" s="9" t="str">
+        <x:v>Owner</x:v>
+      </x:c>
+      <x:c r="C3" s="9" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D3" s="9" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="E3" s="9" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F3" s="9" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G3" s="9" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H3" s="9" t="n">
+        <x:f>ROUND(((E3+F3)*2-G3)/2,1)</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="I3" s="9" t="str">
+        <x:f>IF(H3&gt;=7,"Start",IF(H3&gt;=5,"Test","Skip"))</x:f>
+        <x:v>Test</x:v>
+      </x:c>
+      <x:c r="J3" s="9" t="str">
+        <x:v>投稿テーマだけ人間が決める</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="33" hidden="0" customHeight="1">
+      <x:c r="A4" s="9" t="str">
+        <x:v>商品説明文の改善</x:v>
+      </x:c>
+      <x:c r="B4" s="9" t="str">
+        <x:v>Owner</x:v>
+      </x:c>
+      <x:c r="C4" s="9" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D4" s="9" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E4" s="9" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F4" s="9" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G4" s="9" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H4" s="9" t="n">
+        <x:f>ROUND(((E4+F4)*2-G4)/2,1)</x:f>
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="I4" s="9" t="str">
+        <x:f>IF(H4&gt;=7,"Start",IF(H4&gt;=5,"Test","Skip"))</x:f>
+        <x:v>Start</x:v>
+      </x:c>
+      <x:c r="J4" s="9" t="str">
+        <x:v>実物と違う表現を削る</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="33" hidden="0" customHeight="1">
+      <x:c r="A5" s="9" t="str">
+        <x:v>ブログ記事の構成作成</x:v>
+      </x:c>
+      <x:c r="B5" s="9" t="str">
+        <x:v>Owner</x:v>
+      </x:c>
+      <x:c r="C5" s="9" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D5" s="9" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="E5" s="9" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F5" s="9" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G5" s="9" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H5" s="9" t="n">
+        <x:f>ROUND(((E5+F5)*2-G5)/2,1)</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="I5" s="9" t="str">
+        <x:f>IF(H5&gt;=7,"Start",IF(H5&gt;=5,"Test","Skip"))</x:f>
+        <x:v>Test</x:v>
+      </x:c>
+      <x:c r="J5" s="9" t="str">
+        <x:v>一次情報確認が必要</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="33" hidden="0" customHeight="1">
+      <x:c r="A6" s="9" t="str">
+        <x:v>請求前の確認</x:v>
+      </x:c>
+      <x:c r="B6" s="9" t="str">
+        <x:v>Owner</x:v>
+      </x:c>
+      <x:c r="C6" s="9" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D6" s="9" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="E6" s="9" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F6" s="9" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G6" s="9" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H6" s="9" t="n">
+        <x:f>ROUND(((E6+F6)*2-G6)/2,1)</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="I6" s="9" t="str">
+        <x:f>IF(H6&gt;=7,"Start",IF(H6&gt;=5,"Test","Skip"))</x:f>
+        <x:v>Test</x:v>
+      </x:c>
+      <x:c r="J6" s="9" t="str">
+        <x:v>金額は必ず人間確認</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="33" hidden="0" customHeight="1">
+      <x:c r="A7" s="9" t="str">
+        <x:v>顧客レビュー返信</x:v>
+      </x:c>
+      <x:c r="B7" s="9" t="str">
+        <x:v>Owner</x:v>
+      </x:c>
+      <x:c r="C7" s="9" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D7" s="9" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E7" s="9" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F7" s="9" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G7" s="9" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H7" s="9" t="n">
+        <x:f>ROUND(((E7+F7)*2-G7)/2,1)</x:f>
+        <x:v>5.5</x:v>
+      </x:c>
+      <x:c r="I7" s="9" t="str">
+        <x:f>IF(H7&gt;=7,"Start",IF(H7&gt;=5,"Test","Skip"))</x:f>
+        <x:v>Test</x:v>
+      </x:c>
+      <x:c r="J7" s="9" t="str">
+        <x:v>事実関係を確認</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="33" hidden="0" customHeight="1">
+      <x:c r="A8" s="9" t="str">
+        <x:v>競合記事リサーチ</x:v>
+      </x:c>
+      <x:c r="B8" s="9" t="str">
+        <x:v>Owner</x:v>
+      </x:c>
+      <x:c r="C8" s="9" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D8" s="9" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="E8" s="9" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F8" s="9" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G8" s="9" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H8" s="9" t="n">
+        <x:f>ROUND(((E8+F8)*2-G8)/2,1)</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="I8" s="9" t="str">
+        <x:f>IF(H8&gt;=7,"Start",IF(H8&gt;=5,"Test","Skip"))</x:f>
+        <x:v>Test</x:v>
+      </x:c>
+      <x:c r="J8" s="9" t="str">
+        <x:v>出典を残す</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="33" hidden="0" customHeight="1">
+      <x:c r="A9" s="9" t="str">
+        <x:v>月次改善レポート</x:v>
+      </x:c>
+      <x:c r="B9" s="9" t="str">
+        <x:v>Owner</x:v>
+      </x:c>
+      <x:c r="C9" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D9" s="9" t="n">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="E9" s="9" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F9" s="9" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G9" s="9" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H9" s="9" t="n">
+        <x:f>ROUND(((E9+F9)*2-G9)/2,1)</x:f>
+        <x:v>7.5</x:v>
+      </x:c>
+      <x:c r="I9" s="9" t="str">
+        <x:f>IF(H9&gt;=7,"Start",IF(H9&gt;=5,"Test","Skip"))</x:f>
+        <x:v>Start</x:v>
+      </x:c>
+      <x:c r="J9" s="9" t="str">
+        <x:v>数値入力は人間</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="33" hidden="0" customHeight="1">
+      <x:c r="A10" s="9" t="str">
+        <x:v>FAQ更新</x:v>
+      </x:c>
+      <x:c r="B10" s="9" t="str">
+        <x:v>Owner</x:v>
+      </x:c>
+      <x:c r="C10" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D10" s="9" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="E10" s="9" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F10" s="9" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G10" s="9" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H10" s="9" t="n">
+        <x:f>ROUND(((E10+F10)*2-G10)/2,1)</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="I10" s="9" t="str">
+        <x:f>IF(H10&gt;=7,"Start",IF(H10&gt;=5,"Test","Skip"))</x:f>
+        <x:v>Test</x:v>
+      </x:c>
+      <x:c r="J10" s="9" t="str">
+        <x:v>重複を整理</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="33" hidden="0" customHeight="1">
+      <x:c r="A11" s="9" t="str">
+        <x:v>営業メール下書き</x:v>
+      </x:c>
+      <x:c r="B11" s="9" t="str">
+        <x:v>Owner</x:v>
+      </x:c>
+      <x:c r="C11" s="9" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D11" s="9" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E11" s="9" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F11" s="9" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G11" s="9" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H11" s="9" t="n">
+        <x:f>ROUND(((E11+F11)*2-G11)/2,1)</x:f>
+        <x:v>5.5</x:v>
+      </x:c>
+      <x:c r="I11" s="9" t="str">
+        <x:f>IF(H11&gt;=7,"Start",IF(H11&gt;=5,"Test","Skip"))</x:f>
+        <x:v>Test</x:v>
+      </x:c>
+      <x:c r="J11" s="9" t="str">
+        <x:v>送信前承認</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="24.899999618530273" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="13.59000015258789" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="16.149999618530273" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="12.920000076293945" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="10.5" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="12.25" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="10.899999618530273" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="33" hidden="0" customHeight="1">
+      <x:c r="A1" s="13" t="str">
+        <x:v>Task</x:v>
+      </x:c>
+      <x:c r="B1" s="13" t="str">
+        <x:v>Hours / Month</x:v>
+      </x:c>
+      <x:c r="C1" s="13" t="str">
+        <x:v>Hourly Value JPY</x:v>
+      </x:c>
+      <x:c r="D1" s="13" t="str">
+        <x:v>Expected Reduction</x:v>
+      </x:c>
+      <x:c r="E1" s="13" t="str">
+        <x:v>Value Saved JPY</x:v>
+      </x:c>
+      <x:c r="F1" s="13" t="str">
+        <x:v>Tool Cost JPY</x:v>
+      </x:c>
+      <x:c r="G1" s="13" t="str">
+        <x:v>Net Impact JPY</x:v>
+      </x:c>
+      <x:c r="H1" s="13" t="str">
+        <x:v>Decision</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="33" hidden="0" customHeight="1">
+      <x:c r="A2" s="9" t="str">
+        <x:v>問い合わせ返信の下書き</x:v>
+      </x:c>
+      <x:c r="B2" s="14" t="n">
+        <x:f>XLOOKUP(A2,'Task Inventory'!A:A,'Task Inventory'!C:C)*XLOOKUP(A2,'Task Inventory'!A:A,'Task Inventory'!D:D)*4/60</x:f>
+        <x:v>5.333333333333333</x:v>
+      </x:c>
+      <x:c r="C2" s="15" t="n">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="D2" s="16" t="n">
+        <x:v>0.35</x:v>
+      </x:c>
+      <x:c r="E2" s="15" t="n">
+        <x:f>B2*C2*D2</x:f>
+        <x:v>3733.333333333333</x:v>
+      </x:c>
+      <x:c r="F2" s="15" t="n">
+        <x:v>3000</x:v>
+      </x:c>
+      <x:c r="G2" s="15" t="n">
+        <x:f>ROUND(E2-F2,0)</x:f>
+        <x:v>733</x:v>
+      </x:c>
+      <x:c r="H2" s="9" t="str">
+        <x:f>IF(G2&gt;0,"Worth testing","Wait")</x:f>
+        <x:v>Worth testing</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="33" hidden="0" customHeight="1">
+      <x:c r="A3" s="9" t="str">
+        <x:v>SNS投稿案の作成</x:v>
+      </x:c>
+      <x:c r="B3" s="14" t="n">
+        <x:f>XLOOKUP(A3,'Task Inventory'!A:A,'Task Inventory'!C:C)*XLOOKUP(A3,'Task Inventory'!A:A,'Task Inventory'!D:D)*4/60</x:f>
+        <x:v>6.666666666666667</x:v>
+      </x:c>
+      <x:c r="C3" s="15" t="n">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="D3" s="16" t="n">
+        <x:v>0.45</x:v>
+      </x:c>
+      <x:c r="E3" s="15" t="n">
+        <x:f>B3*C3*D3</x:f>
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="F3" s="15" t="n">
+        <x:v>3000</x:v>
+      </x:c>
+      <x:c r="G3" s="15" t="n">
+        <x:f>ROUND(E3-F3,0)</x:f>
+        <x:v>3000</x:v>
+      </x:c>
+      <x:c r="H3" s="9" t="str">
+        <x:f>IF(G3&gt;0,"Worth testing","Wait")</x:f>
+        <x:v>Worth testing</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="33" hidden="0" customHeight="1">
+      <x:c r="A4" s="9" t="str">
+        <x:v>商品説明文の改善</x:v>
+      </x:c>
+      <x:c r="B4" s="14" t="n">
+        <x:f>XLOOKUP(A4,'Task Inventory'!A:A,'Task Inventory'!C:C)*XLOOKUP(A4,'Task Inventory'!A:A,'Task Inventory'!D:D)*4/60</x:f>
+        <x:v>6.4</x:v>
+      </x:c>
+      <x:c r="C4" s="15" t="n">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="D4" s="16" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="E4" s="15" t="n">
+        <x:f>B4*C4*D4</x:f>
+        <x:v>5120</x:v>
+      </x:c>
+      <x:c r="F4" s="15" t="n">
+        <x:v>3000</x:v>
+      </x:c>
+      <x:c r="G4" s="15" t="n">
+        <x:f>ROUND(E4-F4,0)</x:f>
+        <x:v>2120</x:v>
+      </x:c>
+      <x:c r="H4" s="9" t="str">
+        <x:f>IF(G4&gt;0,"Worth testing","Wait")</x:f>
+        <x:v>Worth testing</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="33" hidden="0" customHeight="1">
+      <x:c r="A5" s="9" t="str">
+        <x:v>競合記事リサーチ</x:v>
+      </x:c>
+      <x:c r="B5" s="14" t="n">
+        <x:f>XLOOKUP(A5,'Task Inventory'!A:A,'Task Inventory'!C:C)*XLOOKUP(A5,'Task Inventory'!A:A,'Task Inventory'!D:D)*4/60</x:f>
+        <x:v>5.333333333333333</x:v>
+      </x:c>
+      <x:c r="C5" s="15" t="n">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="D5" s="16" t="n">
+        <x:v>0.35</x:v>
+      </x:c>
+      <x:c r="E5" s="15" t="n">
+        <x:f>B5*C5*D5</x:f>
+        <x:v>3733.333333333333</x:v>
+      </x:c>
+      <x:c r="F5" s="15" t="n">
+        <x:v>3000</x:v>
+      </x:c>
+      <x:c r="G5" s="15" t="n">
+        <x:f>ROUND(E5-F5,0)</x:f>
+        <x:v>733</x:v>
+      </x:c>
+      <x:c r="H5" s="9" t="str">
+        <x:f>IF(G5&gt;0,"Worth testing","Wait")</x:f>
+        <x:v>Worth testing</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="33" hidden="0" customHeight="1">
+      <x:c r="A6" s="9" t="str">
+        <x:v>月次改善レポート</x:v>
+      </x:c>
+      <x:c r="B6" s="14" t="n">
+        <x:f>XLOOKUP(A6,'Task Inventory'!A:A,'Task Inventory'!C:C)*XLOOKUP(A6,'Task Inventory'!A:A,'Task Inventory'!D:D)*4/60</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C6" s="15" t="n">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="D6" s="16" t="n">
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="E6" s="15" t="n">
+        <x:f>B6*C6*D6</x:f>
+        <x:v>3600</x:v>
+      </x:c>
+      <x:c r="F6" s="15" t="n">
+        <x:v>3000</x:v>
+      </x:c>
+      <x:c r="G6" s="15" t="n">
+        <x:f>ROUND(E6-F6,0)</x:f>
+        <x:v>600</x:v>
+      </x:c>
+      <x:c r="H6" s="9" t="str">
+        <x:f>IF(G6&gt;0,"Worth testing","Wait")</x:f>
+        <x:v>Worth testing</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="4.039999961853027" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="23.549999237060547" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="23.549999237060547" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="23.549999237060547" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="23.549999237060547" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="23.549999237060547" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="33" hidden="0" customHeight="1">
+      <x:c r="A1" s="13" t="str">
+        <x:v>Rank</x:v>
+      </x:c>
+      <x:c r="B1" s="13" t="str">
+        <x:v>Best First Task</x:v>
+      </x:c>
+      <x:c r="C1" s="13" t="str">
+        <x:v>Priority</x:v>
+      </x:c>
+      <x:c r="D1" s="13" t="str">
+        <x:v>Monthly Net Impact</x:v>
+      </x:c>
+      <x:c r="E1" s="13" t="str">
+        <x:v>Recommended Tool Stack</x:v>
+      </x:c>
+      <x:c r="F1" s="13" t="str">
+        <x:v>Next 7 Days</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="33" hidden="0" customHeight="1">
+      <x:c r="A2" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B2" s="9" t="str">
+        <x:f>INDEX('Task Inventory'!$A$2:$A$11,MATCH(LARGE('Task Inventory'!$H$2:$H$11,A2),'Task Inventory'!$H$2:$H$11,0))</x:f>
+        <x:v>商品説明文の改善</x:v>
+      </x:c>
+      <x:c r="C2" s="9" t="str">
+        <x:f>XLOOKUP(B2,'Task Inventory'!A:A,'Task Inventory'!I:I)</x:f>
+        <x:v>Start</x:v>
+      </x:c>
+      <x:c r="D2" s="15" t="n">
+        <x:f>IFERROR(ROUND(XLOOKUP(B2,'ROI Calculator'!A:A,'ROI Calculator'!G:G),0),"")</x:f>
+        <x:v>2120</x:v>
+      </x:c>
+      <x:c r="E2" s="9" t="str">
+        <x:v>ChatGPT or Claude + spreadsheet</x:v>
+      </x:c>
+      <x:c r="F2" s="9" t="str">
+        <x:v>1つの作業だけで試す</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="33" hidden="0" customHeight="1">
+      <x:c r="A3" s="9" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B3" s="9" t="str">
+        <x:f>INDEX('Task Inventory'!$A$2:$A$11,MATCH(LARGE('Task Inventory'!$H$2:$H$11,A3),'Task Inventory'!$H$2:$H$11,0))</x:f>
+        <x:v>月次改善レポート</x:v>
+      </x:c>
+      <x:c r="C3" s="9" t="str">
+        <x:f>XLOOKUP(B3,'Task Inventory'!A:A,'Task Inventory'!I:I)</x:f>
+        <x:v>Start</x:v>
+      </x:c>
+      <x:c r="D3" s="15" t="n">
+        <x:f>IFERROR(ROUND(XLOOKUP(B3,'ROI Calculator'!A:A,'ROI Calculator'!G:G),0),"")</x:f>
+        <x:v>600</x:v>
+      </x:c>
+      <x:c r="E3" s="9" t="str">
+        <x:v>ChatGPT + Zapier</x:v>
+      </x:c>
+      <x:c r="F3" s="9" t="str">
+        <x:v>自動送信はしない</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="33" hidden="0" customHeight="1">
+      <x:c r="A4" s="9" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B4" s="9" t="str">
+        <x:f>INDEX('Task Inventory'!$A$2:$A$11,MATCH(LARGE('Task Inventory'!$H$2:$H$11,A4),'Task Inventory'!$H$2:$H$11,0))</x:f>
+        <x:v>問い合わせ返信の下書き</x:v>
+      </x:c>
+      <x:c r="C4" s="9" t="str">
+        <x:f>XLOOKUP(B4,'Task Inventory'!A:A,'Task Inventory'!I:I)</x:f>
+        <x:v>Test</x:v>
+      </x:c>
+      <x:c r="D4" s="15" t="n">
+        <x:f>IFERROR(ROUND(XLOOKUP(B4,'ROI Calculator'!A:A,'ROI Calculator'!G:G),0),"")</x:f>
+        <x:v>733</x:v>
+      </x:c>
+      <x:c r="E4" s="9" t="str">
+        <x:v>ChatGPT + Notion/Sheets</x:v>
+      </x:c>
+      <x:c r="F4" s="9" t="str">
+        <x:v>入力例を3つ作る</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -404,7 +1109,7 @@
       <x:c r="D2" s="9" t="str">
         <x:v>Research, writing, ideation</x:v>
       </x:c>
-      <x:c r="E2" s="14" t="n">
+      <x:c r="E2" s="15" t="n">
         <x:v>3000</x:v>
       </x:c>
       <x:c r="F2" s="9" t="str">
@@ -440,7 +1145,7 @@
       <x:c r="D3" s="9" t="str">
         <x:v>Search-connected research</x:v>
       </x:c>
-      <x:c r="E3" s="14" t="n">
+      <x:c r="E3" s="15" t="n">
         <x:v>2900</x:v>
       </x:c>
       <x:c r="F3" s="9" t="str">
@@ -476,7 +1181,7 @@
       <x:c r="D4" s="9" t="str">
         <x:v>Long document writing</x:v>
       </x:c>
-      <x:c r="E4" s="14" t="n">
+      <x:c r="E4" s="15" t="n">
         <x:v>3000</x:v>
       </x:c>
       <x:c r="F4" s="9" t="str">
@@ -512,7 +1217,7 @@
       <x:c r="D5" s="9" t="str">
         <x:v>Marketing copy and brand content</x:v>
       </x:c>
-      <x:c r="E5" s="14" t="n">
+      <x:c r="E5" s="15" t="n">
         <x:v>9000</x:v>
       </x:c>
       <x:c r="F5" s="9" t="str">
@@ -548,7 +1253,7 @@
       <x:c r="D6" s="9" t="str">
         <x:v>Blog and ad copy</x:v>
       </x:c>
-      <x:c r="E6" s="14" t="n">
+      <x:c r="E6" s="15" t="n">
         <x:v>3000</x:v>
       </x:c>
       <x:c r="F6" s="9" t="str">
@@ -584,7 +1289,7 @@
       <x:c r="D7" s="9" t="str">
         <x:v>SEO content optimization</x:v>
       </x:c>
-      <x:c r="E7" s="14" t="n">
+      <x:c r="E7" s="15" t="n">
         <x:v>13000</x:v>
       </x:c>
       <x:c r="F7" s="9" t="str">
@@ -620,7 +1325,7 @@
       <x:c r="D8" s="9" t="str">
         <x:v>Workflow automation</x:v>
       </x:c>
-      <x:c r="E8" s="14" t="n">
+      <x:c r="E8" s="15" t="n">
         <x:v>3000</x:v>
       </x:c>
       <x:c r="F8" s="9" t="str">
@@ -656,7 +1361,7 @@
       <x:c r="D9" s="9" t="str">
         <x:v>Knowledge base and docs</x:v>
       </x:c>
-      <x:c r="E9" s="14" t="n">
+      <x:c r="E9" s="15" t="n">
         <x:v>1500</x:v>
       </x:c>
       <x:c r="F9" s="9" t="str">
@@ -684,7 +1389,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -728,22 +1433,22 @@
       <x:c r="A2" s="9" t="str">
         <x:v>SNS投稿を週5本作る</x:v>
       </x:c>
-      <x:c r="B2" s="15" t="n">
+      <x:c r="B2" s="17" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="C2" s="15" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="D2" s="15" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="E2" s="15" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="F2" s="15" t="n">
+      <x:c r="C2" s="17" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D2" s="17" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E2" s="17" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F2" s="17" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="G2" s="15" t="n">
+      <x:c r="G2" s="17" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="H2" s="9" t="str">
@@ -755,22 +1460,22 @@
       <x:c r="A3" s="9" t="str">
         <x:v>問い合わせ返信の下書き</x:v>
       </x:c>
-      <x:c r="B3" s="15" t="n">
+      <x:c r="B3" s="17" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="C3" s="15" t="n">
+      <x:c r="C3" s="17" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="D3" s="15" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="E3" s="15" t="n">
+      <x:c r="D3" s="17" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E3" s="17" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="F3" s="15" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="G3" s="15" t="n">
+      <x:c r="F3" s="17" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G3" s="17" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="H3" s="9" t="str">
@@ -782,22 +1487,22 @@
       <x:c r="A4" s="9" t="str">
         <x:v>ブログ記事の構成作成</x:v>
       </x:c>
-      <x:c r="B4" s="15" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C4" s="15" t="n">
+      <x:c r="B4" s="17" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C4" s="17" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="D4" s="15" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="E4" s="15" t="n">
+      <x:c r="D4" s="17" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E4" s="17" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="F4" s="15" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="G4" s="15" t="n">
+      <x:c r="F4" s="17" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G4" s="17" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="H4" s="9" t="str">
@@ -809,22 +1514,22 @@
       <x:c r="A5" s="9" t="str">
         <x:v>SEOリライト</x:v>
       </x:c>
-      <x:c r="B5" s="15" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C5" s="15" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D5" s="15" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="E5" s="15" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="F5" s="15" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="G5" s="15" t="n">
+      <x:c r="B5" s="17" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C5" s="17" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D5" s="17" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E5" s="17" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F5" s="17" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G5" s="17" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="H5" s="9" t="str">
@@ -836,22 +1541,22 @@
       <x:c r="A6" s="9" t="str">
         <x:v>請求/顧客管理の自動化</x:v>
       </x:c>
-      <x:c r="B6" s="15" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C6" s="15" t="n">
+      <x:c r="B6" s="17" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C6" s="17" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="D6" s="15" t="n">
+      <x:c r="D6" s="17" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="E6" s="15" t="n">
+      <x:c r="E6" s="17" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="F6" s="15" t="n">
+      <x:c r="F6" s="17" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="G6" s="15" t="n">
+      <x:c r="G6" s="17" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="H6" s="9" t="str">
@@ -863,22 +1568,22 @@
       <x:c r="A7" s="9" t="str">
         <x:v>商品説明文の改善</x:v>
       </x:c>
-      <x:c r="B7" s="15" t="n">
+      <x:c r="B7" s="17" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="C7" s="15" t="n">
+      <x:c r="C7" s="17" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="D7" s="15" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="E7" s="15" t="n">
+      <x:c r="D7" s="17" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E7" s="17" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="F7" s="15" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="G7" s="15" t="n">
+      <x:c r="F7" s="17" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G7" s="17" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="H7" s="9" t="str">
@@ -890,22 +1595,22 @@
       <x:c r="A8" s="9" t="str">
         <x:v>社内手順書の整備</x:v>
       </x:c>
-      <x:c r="B8" s="15" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C8" s="15" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="D8" s="15" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="E8" s="15" t="n">
+      <x:c r="B8" s="17" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C8" s="17" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D8" s="17" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E8" s="17" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="F8" s="15" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="G8" s="15" t="n">
+      <x:c r="F8" s="17" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G8" s="17" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="H8" s="9" t="str">
@@ -915,46 +1620,46 @@
     </x:row>
     <x:row r="9" ht="33" hidden="0" customHeight="1">
       <x:c r="A9" s="9"/>
-      <x:c r="B9" s="15"/>
-      <x:c r="C9" s="15"/>
-      <x:c r="D9" s="15"/>
-      <x:c r="E9" s="15"/>
-      <x:c r="F9" s="15"/>
-      <x:c r="G9" s="15"/>
+      <x:c r="B9" s="17"/>
+      <x:c r="C9" s="17"/>
+      <x:c r="D9" s="17"/>
+      <x:c r="E9" s="17"/>
+      <x:c r="F9" s="17"/>
+      <x:c r="G9" s="17"/>
       <x:c r="H9" s="9"/>
     </x:row>
     <x:row r="10" ht="33" hidden="0" customHeight="1">
       <x:c r="A10" s="9" t="str">
         <x:v>Weighted Total</x:v>
       </x:c>
-      <x:c r="B10" s="15" t="str"/>
-      <x:c r="C10" s="15" t="str"/>
-      <x:c r="D10" s="15" t="str"/>
-      <x:c r="E10" s="15" t="str"/>
-      <x:c r="F10" s="15" t="str"/>
-      <x:c r="G10" s="15" t="str"/>
+      <x:c r="B10" s="17" t="str"/>
+      <x:c r="C10" s="17" t="str"/>
+      <x:c r="D10" s="17" t="str"/>
+      <x:c r="E10" s="17" t="str"/>
+      <x:c r="F10" s="17" t="str"/>
+      <x:c r="G10" s="17" t="str"/>
       <x:c r="H10" s="9" t="str"/>
     </x:row>
     <x:row r="11" ht="33" hidden="0" customHeight="1">
       <x:c r="A11" s="9"/>
-      <x:c r="B11" s="15"/>
-      <x:c r="C11" s="15" t="n">
+      <x:c r="B11" s="17"/>
+      <x:c r="C11" s="17" t="n">
         <x:f>SUMPRODUCT($B$2:$B$8,C2:C8)</x:f>
         <x:v>119</x:v>
       </x:c>
-      <x:c r="D11" s="15" t="n">
+      <x:c r="D11" s="17" t="n">
         <x:f>SUMPRODUCT($B$2:$B$8,D2:D8)</x:f>
         <x:v>100</x:v>
       </x:c>
-      <x:c r="E11" s="15" t="n">
+      <x:c r="E11" s="17" t="n">
         <x:f>SUMPRODUCT($B$2:$B$8,E2:E8)</x:f>
         <x:v>125</x:v>
       </x:c>
-      <x:c r="F11" s="15" t="n">
+      <x:c r="F11" s="17" t="n">
         <x:f>SUMPRODUCT($B$2:$B$8,F2:F8)</x:f>
         <x:v>105</x:v>
       </x:c>
-      <x:c r="G11" s="15" t="n">
+      <x:c r="G11" s="17" t="n">
         <x:f>SUMPRODUCT($B$2:$B$8,G2:G8)</x:f>
         <x:v>101</x:v>
       </x:c>
@@ -965,7 +1670,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -1190,7 +1895,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -1303,7 +2008,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>

</xml_diff>

<commit_message>
Add industry presets and 7 day AI plan
</commit_message>
<xml_diff>
--- a/products/AI_Tool_Selection_Checklist_v0.1.xlsx
+++ b/products/AI_Tool_Selection_Checklist_v0.1.xlsx
@@ -2,15 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start" sheetId="1" r:id="R4cc2e84383bd4c71"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Inventory" sheetId="2" r:id="R6f54f84a0f714638"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROI Calculator" sheetId="3" r:id="R51873790ba8a429b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Summary" sheetId="4" r:id="R76a514304d0c47a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tool Matrix" sheetId="5" r:id="Rc4e00a7ec5644a96"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Use Case Scores" sheetId="6" r:id="R40826377ec9e463a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Automation Recipes" sheetId="7" r:id="R49bb289fc74f44b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt Pack" sheetId="8" r:id="R25a637bba2d04737"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="9" r:id="Rda424072508f41b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start" sheetId="1" r:id="Rcabd814d1d1b4a79"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Inventory" sheetId="2" r:id="R166429c52ec14a1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROI Calculator" sheetId="3" r:id="R59962facd18c4fd2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Summary" sheetId="4" r:id="R8daff00953ab484f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Industry Presets" sheetId="5" r:id="R02ebb989e3c64150"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7 Day Plan" sheetId="6" r:id="R71f9851102794373"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tool Matrix" sheetId="7" r:id="R3513af77d1074e92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Use Case Scores" sheetId="8" r:id="Rf06d17b21c7f4e1b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Automation Recipes" sheetId="9" r:id="R203619a92009426d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt Pack" sheetId="10" r:id="Rc6b952ad86d4406a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="11" r:id="Rb0bd2d7d1d2644e8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -350,6 +352,246 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="13.729999542236328" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="10.09000015258789" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="121.12999725341797" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="29.610000610351562" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="33" hidden="0" customHeight="1">
+      <x:c r="A1" s="13" t="str">
+        <x:v>Prompt Name</x:v>
+      </x:c>
+      <x:c r="B1" s="13" t="str">
+        <x:v>Use Case</x:v>
+      </x:c>
+      <x:c r="C1" s="13" t="str">
+        <x:v>Prompt</x:v>
+      </x:c>
+      <x:c r="D1" s="13" t="str">
+        <x:v>Check Before Use</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="33" hidden="0" customHeight="1">
+      <x:c r="A2" s="9" t="str">
+        <x:v>AIツール比較</x:v>
+      </x:c>
+      <x:c r="B2" s="9" t="str">
+        <x:v>導入検討</x:v>
+      </x:c>
+      <x:c r="C2" s="9" t="str">
+        <x:v>あなたは小規模事業者向けの業務改善担当です。次の用途、予算、既存ツールをもとにAIツール候補を比較し、導入しない選択肢も含めて提案してください。</x:v>
+      </x:c>
+      <x:c r="D2" s="9" t="str">
+        <x:v>価格と規約を公式サイトで確認</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="33" hidden="0" customHeight="1">
+      <x:c r="A3" s="9" t="str">
+        <x:v>商品説明改善</x:v>
+      </x:c>
+      <x:c r="B3" s="9" t="str">
+        <x:v>EC/フリマ</x:v>
+      </x:c>
+      <x:c r="C3" s="9" t="str">
+        <x:v>次の商品情報から、誇張せず、購入前の不安を減らす商品説明文、見出し、FAQを作ってください。事実不明な点は質問として返してください。</x:v>
+      </x:c>
+      <x:c r="D3" s="9" t="str">
+        <x:v>実物と違う表現を削除</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="33" hidden="0" customHeight="1">
+      <x:c r="A4" s="9" t="str">
+        <x:v>問い合わせ返信</x:v>
+      </x:c>
+      <x:c r="B4" s="9" t="str">
+        <x:v>顧客対応</x:v>
+      </x:c>
+      <x:c r="C4" s="9" t="str">
+        <x:v>次の問い合わせに対し、丁寧で短い返信案を3パターン作ってください。約束できない内容は避け、確認事項を箇条書きにしてください。</x:v>
+      </x:c>
+      <x:c r="D4" s="9" t="str">
+        <x:v>送信前に個人情報と条件を確認</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="33" hidden="0" customHeight="1">
+      <x:c r="A5" s="9" t="str">
+        <x:v>SNS投稿案</x:v>
+      </x:c>
+      <x:c r="B5" s="9" t="str">
+        <x:v>マーケ</x:v>
+      </x:c>
+      <x:c r="C5" s="9" t="str">
+        <x:v>次のテーマから、売り込みすぎないSNS投稿案を10本作ってください。各投稿に狙い、想定読者、CTAを付けてください。</x:v>
+      </x:c>
+      <x:c r="D5" s="9" t="str">
+        <x:v>断定表現と炎上リスクを確認</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="33" hidden="0" customHeight="1">
+      <x:c r="A6" s="9" t="str">
+        <x:v>記事構成</x:v>
+      </x:c>
+      <x:c r="B6" s="9" t="str">
+        <x:v>SEO/ブログ</x:v>
+      </x:c>
+      <x:c r="C6" s="9" t="str">
+        <x:v>次のキーワードについて、検索者の悩み、記事構成、見出し、入れるべき一次情報、避けるべき誇大表現を整理してください。</x:v>
+      </x:c>
+      <x:c r="D6" s="9" t="str">
+        <x:v>一次情報リンクを追加</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="33" hidden="0" customHeight="1">
+      <x:c r="A7" s="9" t="str">
+        <x:v>業務自動化分解</x:v>
+      </x:c>
+      <x:c r="B7" s="9" t="str">
+        <x:v>Zapier/Make</x:v>
+      </x:c>
+      <x:c r="C7" s="9" t="str">
+        <x:v>次の手作業を、トリガー、入力、AI処理、出力、人間確認、失敗時対応に分解してください。</x:v>
+      </x:c>
+      <x:c r="D7" s="9" t="str">
+        <x:v>自動送信や課金処理は承認制にする</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="13.319999694824219" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22.209999084472656" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18.56999969482422" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="10.5" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="33" hidden="0" customHeight="1">
+      <x:c r="A1" s="13" t="str">
+        <x:v>Source</x:v>
+      </x:c>
+      <x:c r="B1" s="13" t="str">
+        <x:v>URL</x:v>
+      </x:c>
+      <x:c r="C1" s="13" t="str">
+        <x:v>Purpose</x:v>
+      </x:c>
+      <x:c r="D1" s="13" t="str">
+        <x:v>Last Checked</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="33" hidden="0" customHeight="1">
+      <x:c r="A2" s="9" t="str">
+        <x:v>OpenAI ChatGPT</x:v>
+      </x:c>
+      <x:c r="B2" s="9" t="str">
+        <x:v>https://openai.com/chatgpt</x:v>
+      </x:c>
+      <x:c r="C2" s="9" t="str">
+        <x:v>General AI candidate</x:v>
+      </x:c>
+      <x:c r="D2" s="9" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="33" hidden="0" customHeight="1">
+      <x:c r="A3" s="9" t="str">
+        <x:v>Google Gemini</x:v>
+      </x:c>
+      <x:c r="B3" s="9" t="str">
+        <x:v>https://gemini.google.com</x:v>
+      </x:c>
+      <x:c r="C3" s="9" t="str">
+        <x:v>General AI candidate</x:v>
+      </x:c>
+      <x:c r="D3" s="9" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="33" hidden="0" customHeight="1">
+      <x:c r="A4" s="9" t="str">
+        <x:v>Claude</x:v>
+      </x:c>
+      <x:c r="B4" s="9" t="str">
+        <x:v>https://claude.ai</x:v>
+      </x:c>
+      <x:c r="C4" s="9" t="str">
+        <x:v>General AI candidate</x:v>
+      </x:c>
+      <x:c r="D4" s="9" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="33" hidden="0" customHeight="1">
+      <x:c r="A5" s="9" t="str">
+        <x:v>Jasper</x:v>
+      </x:c>
+      <x:c r="B5" s="9" t="str">
+        <x:v>https://www.jasper.ai</x:v>
+      </x:c>
+      <x:c r="C5" s="9" t="str">
+        <x:v>Marketing AI candidate</x:v>
+      </x:c>
+      <x:c r="D5" s="9" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="33" hidden="0" customHeight="1">
+      <x:c r="A6" s="9" t="str">
+        <x:v>Writesonic</x:v>
+      </x:c>
+      <x:c r="B6" s="9" t="str">
+        <x:v>https://writesonic.com</x:v>
+      </x:c>
+      <x:c r="C6" s="9" t="str">
+        <x:v>Marketing AI candidate</x:v>
+      </x:c>
+      <x:c r="D6" s="9" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="33" hidden="0" customHeight="1">
+      <x:c r="A7" s="9" t="str">
+        <x:v>Surfer SEO</x:v>
+      </x:c>
+      <x:c r="B7" s="9" t="str">
+        <x:v>https://surferseo.com</x:v>
+      </x:c>
+      <x:c r="C7" s="9" t="str">
+        <x:v>SEO candidate</x:v>
+      </x:c>
+      <x:c r="D7" s="9" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="33" hidden="0" customHeight="1">
+      <x:c r="A8" s="9" t="str">
+        <x:v>Zapier</x:v>
+      </x:c>
+      <x:c r="B8" s="9" t="str">
+        <x:v>https://zapier.com</x:v>
+      </x:c>
+      <x:c r="C8" s="9" t="str">
+        <x:v>Automation candidate</x:v>
+      </x:c>
+      <x:c r="D8" s="9" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
@@ -1048,6 +1290,540 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
+    <x:col min="1" max="1" width="18.170000076293945" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24.899999618530273" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="24.899999618530273" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="24.899999618530273" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="24.899999618530273" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="24.899999618530273" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="24.899999618530273" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="24.899999618530273" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="33" hidden="0" customHeight="1">
+      <x:c r="A1" s="13" t="str">
+        <x:v>Business Type</x:v>
+      </x:c>
+      <x:c r="B1" s="13" t="str">
+        <x:v>Best First Task</x:v>
+      </x:c>
+      <x:c r="C1" s="13" t="str">
+        <x:v>Why It Matters</x:v>
+      </x:c>
+      <x:c r="D1" s="13" t="str">
+        <x:v>Suggested AI Step</x:v>
+      </x:c>
+      <x:c r="E1" s="13" t="str">
+        <x:v>Keep Human Approval For</x:v>
+      </x:c>
+      <x:c r="F1" s="13" t="str">
+        <x:v>Starter Prompt</x:v>
+      </x:c>
+      <x:c r="G1" s="13" t="str">
+        <x:v>Expected Signal</x:v>
+      </x:c>
+      <x:c r="H1" s="13" t="str">
+        <x:v>Avoid</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="33" hidden="0" customHeight="1">
+      <x:c r="A2" s="9" t="str">
+        <x:v>EC / フリマ</x:v>
+      </x:c>
+      <x:c r="B2" s="9" t="str">
+        <x:v>商品説明文の改善</x:v>
+      </x:c>
+      <x:c r="C2" s="9" t="str">
+        <x:v>出品作業が多く、文章の差が購入判断に出やすい</x:v>
+      </x:c>
+      <x:c r="D2" s="9" t="str">
+        <x:v>特徴から見出し・説明文・FAQを生成</x:v>
+      </x:c>
+      <x:c r="E2" s="9" t="str">
+        <x:v>状態、傷、サイズ、発送条件</x:v>
+      </x:c>
+      <x:c r="F2" s="9" t="str">
+        <x:v>この商品情報から、誇張せず購入前の不安を減らす説明文を作ってください。</x:v>
+      </x:c>
+      <x:c r="G2" s="9" t="str">
+        <x:v>閲覧数、保存数、質問数</x:v>
+      </x:c>
+      <x:c r="H2" s="9" t="str">
+        <x:v>実物と違う表現</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="33" hidden="0" customHeight="1">
+      <x:c r="A3" s="9" t="str">
+        <x:v>美容室 / サロン</x:v>
+      </x:c>
+      <x:c r="B3" s="9" t="str">
+        <x:v>SNS投稿案と予約導線</x:v>
+      </x:c>
+      <x:c r="C3" s="9" t="str">
+        <x:v>投稿ネタ切れと予約導線の弱さが起きやすい</x:v>
+      </x:c>
+      <x:c r="D3" s="9" t="str">
+        <x:v>施術例から投稿文とCTAを作る</x:v>
+      </x:c>
+      <x:c r="E3" s="9" t="str">
+        <x:v>価格、空き枠、ビフォーアフター許可</x:v>
+      </x:c>
+      <x:c r="F3" s="9" t="str">
+        <x:v>次の施術メニューから、予約につながるSNS投稿案を5本作ってください。</x:v>
+      </x:c>
+      <x:c r="G3" s="9" t="str">
+        <x:v>DM数、予約数</x:v>
+      </x:c>
+      <x:c r="H3" s="9" t="str">
+        <x:v>効果保証</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="33" hidden="0" customHeight="1">
+      <x:c r="A4" s="9" t="str">
+        <x:v>飲食店</x:v>
+      </x:c>
+      <x:c r="B4" s="9" t="str">
+        <x:v>口コミ返信と季節メニュー告知</x:v>
+      </x:c>
+      <x:c r="C4" s="9" t="str">
+        <x:v>返信の遅れと告知不足が機会損失になる</x:v>
+      </x:c>
+      <x:c r="D4" s="9" t="str">
+        <x:v>レビュー返信案と投稿案を作る</x:v>
+      </x:c>
+      <x:c r="E4" s="9" t="str">
+        <x:v>事実関係、謝罪、営業日</x:v>
+      </x:c>
+      <x:c r="F4" s="9" t="str">
+        <x:v>次の口コミに対し、丁寧で短い返信を3案作ってください。</x:v>
+      </x:c>
+      <x:c r="G4" s="9" t="str">
+        <x:v>返信率、来店問い合わせ</x:v>
+      </x:c>
+      <x:c r="H4" s="9" t="str">
+        <x:v>過剰な謝罪や断定</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="33" hidden="0" customHeight="1">
+      <x:c r="A5" s="9" t="str">
+        <x:v>士業 / コンサル</x:v>
+      </x:c>
+      <x:c r="B5" s="9" t="str">
+        <x:v>問い合わせ整理</x:v>
+      </x:c>
+      <x:c r="C5" s="9" t="str">
+        <x:v>初回相談前の要件整理に時間がかかる</x:v>
+      </x:c>
+      <x:c r="D5" s="9" t="str">
+        <x:v>相談内容を論点・確認事項に分解</x:v>
+      </x:c>
+      <x:c r="E5" s="9" t="str">
+        <x:v>法的判断、見積、契約条件</x:v>
+      </x:c>
+      <x:c r="F5" s="9" t="str">
+        <x:v>次の問い合わせを、論点、確認事項、返信案に分けてください。</x:v>
+      </x:c>
+      <x:c r="G5" s="9" t="str">
+        <x:v>初回返信時間</x:v>
+      </x:c>
+      <x:c r="H5" s="9" t="str">
+        <x:v>専門判断の自動化</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="33" hidden="0" customHeight="1">
+      <x:c r="A6" s="9" t="str">
+        <x:v>講師 / コーチ</x:v>
+      </x:c>
+      <x:c r="B6" s="9" t="str">
+        <x:v>教材と課題のたたき台</x:v>
+      </x:c>
+      <x:c r="C6" s="9" t="str">
+        <x:v>毎回の教材作成と復習課題が重い</x:v>
+      </x:c>
+      <x:c r="D6" s="9" t="str">
+        <x:v>テーマから構成・例題・宿題案を作る</x:v>
+      </x:c>
+      <x:c r="E6" s="9" t="str">
+        <x:v>受講者レベル、表現、約束範囲</x:v>
+      </x:c>
+      <x:c r="F6" s="9" t="str">
+        <x:v>次のテーマで、初心者向けの30分レッスン構成を作ってください。</x:v>
+      </x:c>
+      <x:c r="G6" s="9" t="str">
+        <x:v>教材作成時間</x:v>
+      </x:c>
+      <x:c r="H6" s="9" t="str">
+        <x:v>成果保証</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="33" hidden="0" customHeight="1">
+      <x:c r="A7" s="9" t="str">
+        <x:v>不動産 / 建築</x:v>
+      </x:c>
+      <x:c r="B7" s="9" t="str">
+        <x:v>物件説明とFAQ</x:v>
+      </x:c>
+      <x:c r="C7" s="9" t="str">
+        <x:v>説明文作成と問い合わせ対応が反復しやすい</x:v>
+      </x:c>
+      <x:c r="D7" s="9" t="str">
+        <x:v>物件情報から説明文・質問回答を作る</x:v>
+      </x:c>
+      <x:c r="E7" s="9" t="str">
+        <x:v>価格、法令、契約条件</x:v>
+      </x:c>
+      <x:c r="F7" s="9" t="str">
+        <x:v>次の物件情報から、事実ベースの紹介文とFAQを作ってください。</x:v>
+      </x:c>
+      <x:c r="G7" s="9" t="str">
+        <x:v>問い合わせ数</x:v>
+      </x:c>
+      <x:c r="H7" s="9" t="str">
+        <x:v>未確認情報</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="33" hidden="0" customHeight="1">
+      <x:c r="A8" s="9" t="str">
+        <x:v>制作会社 / フリーランス</x:v>
+      </x:c>
+      <x:c r="B8" s="9" t="str">
+        <x:v>提案書の初稿</x:v>
+      </x:c>
+      <x:c r="C8" s="9" t="str">
+        <x:v>ヒアリング後の提案書作成が重い</x:v>
+      </x:c>
+      <x:c r="D8" s="9" t="str">
+        <x:v>要件から課題・提案・工程を整理</x:v>
+      </x:c>
+      <x:c r="E8" s="9" t="str">
+        <x:v>納期、金額、責任範囲</x:v>
+      </x:c>
+      <x:c r="F8" s="9" t="str">
+        <x:v>次のヒアリングメモから、提案書の構成と初稿を作ってください。</x:v>
+      </x:c>
+      <x:c r="G8" s="9" t="str">
+        <x:v>提案作成時間</x:v>
+      </x:c>
+      <x:c r="H8" s="9" t="str">
+        <x:v>できない約束</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="33" hidden="0" customHeight="1">
+      <x:c r="A9" s="9" t="str">
+        <x:v>整体 / 治療院</x:v>
+      </x:c>
+      <x:c r="B9" s="9" t="str">
+        <x:v>来院前説明とFAQ</x:v>
+      </x:c>
+      <x:c r="C9" s="9" t="str">
+        <x:v>初回客の不安解消に文章が効く</x:v>
+      </x:c>
+      <x:c r="D9" s="9" t="str">
+        <x:v>症状別の一般的説明と来院案内を作る</x:v>
+      </x:c>
+      <x:c r="E9" s="9" t="str">
+        <x:v>医療的判断、効果表現、禁忌</x:v>
+      </x:c>
+      <x:c r="F9" s="9" t="str">
+        <x:v>次のメニューについて、医療効果を断定せず来院前の不安を減らす説明を作ってください。</x:v>
+      </x:c>
+      <x:c r="G9" s="9" t="str">
+        <x:v>予約前質問数</x:v>
+      </x:c>
+      <x:c r="H9" s="9" t="str">
+        <x:v>診断・治療保証</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="33" hidden="0" customHeight="1">
+      <x:c r="A10" s="9" t="str">
+        <x:v>採用 / 人事</x:v>
+      </x:c>
+      <x:c r="B10" s="9" t="str">
+        <x:v>求人票の改善</x:v>
+      </x:c>
+      <x:c r="C10" s="9" t="str">
+        <x:v>求人票の曖昧さが応募の質を下げる</x:v>
+      </x:c>
+      <x:c r="D10" s="9" t="str">
+        <x:v>仕事内容・魅力・向かない人を整理</x:v>
+      </x:c>
+      <x:c r="E10" s="9" t="str">
+        <x:v>給与、雇用条件、法令表現</x:v>
+      </x:c>
+      <x:c r="F10" s="9" t="str">
+        <x:v>次の求人情報から、誤解が少ない求人票に改善してください。</x:v>
+      </x:c>
+      <x:c r="G10" s="9" t="str">
+        <x:v>応募率、面談率</x:v>
+      </x:c>
+      <x:c r="H10" s="9" t="str">
+        <x:v>条件の盛りすぎ</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="33" hidden="0" customHeight="1">
+      <x:c r="A11" s="9" t="str">
+        <x:v>地域店舗</x:v>
+      </x:c>
+      <x:c r="B11" s="9" t="str">
+        <x:v>Googleビジネス投稿</x:v>
+      </x:c>
+      <x:c r="C11" s="9" t="str">
+        <x:v>更新不足で検索面の魅力が弱くなる</x:v>
+      </x:c>
+      <x:c r="D11" s="9" t="str">
+        <x:v>季節情報から投稿文と写真案を作る</x:v>
+      </x:c>
+      <x:c r="E11" s="9" t="str">
+        <x:v>営業時間、価格、在庫</x:v>
+      </x:c>
+      <x:c r="F11" s="9" t="str">
+        <x:v>次の店舗情報から、Googleビジネスプロフィール用投稿を作ってください。</x:v>
+      </x:c>
+      <x:c r="G11" s="9" t="str">
+        <x:v>電話、経路検索</x:v>
+      </x:c>
+      <x:c r="H11" s="9" t="str">
+        <x:v>古い情報</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="33" hidden="0" customHeight="1">
+      <x:c r="A12" s="9" t="str">
+        <x:v>YouTube / 配信</x:v>
+      </x:c>
+      <x:c r="B12" s="9" t="str">
+        <x:v>タイトルと構成改善</x:v>
+      </x:c>
+      <x:c r="C12" s="9" t="str">
+        <x:v>動画内容はあるが見せ方で損をしやすい</x:v>
+      </x:c>
+      <x:c r="D12" s="9" t="str">
+        <x:v>要点からタイトル・章立て・概要欄を生成</x:v>
+      </x:c>
+      <x:c r="E12" s="9" t="str">
+        <x:v>権利、引用、煽り表現</x:v>
+      </x:c>
+      <x:c r="F12" s="9" t="str">
+        <x:v>次の動画メモから、クリックされやすく誇張しないタイトル案を10個作ってください。</x:v>
+      </x:c>
+      <x:c r="G12" s="9" t="str">
+        <x:v>CTR、視聴維持</x:v>
+      </x:c>
+      <x:c r="H12" s="9" t="str">
+        <x:v>釣りタイトル</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="33" hidden="0" customHeight="1">
+      <x:c r="A13" s="9" t="str">
+        <x:v>バックオフィス</x:v>
+      </x:c>
+      <x:c r="B13" s="9" t="str">
+        <x:v>月次報告の下書き</x:v>
+      </x:c>
+      <x:c r="C13" s="9" t="str">
+        <x:v>毎月似た報告に時間がかかる</x:v>
+      </x:c>
+      <x:c r="D13" s="9" t="str">
+        <x:v>数値から変化点と次アクションを整理</x:v>
+      </x:c>
+      <x:c r="E13" s="9" t="str">
+        <x:v>数値、原因断定、対外表現</x:v>
+      </x:c>
+      <x:c r="F13" s="9" t="str">
+        <x:v>次の月次数値から、変化点、原因仮説、次アクションを整理してください。</x:v>
+      </x:c>
+      <x:c r="G13" s="9" t="str">
+        <x:v>報告作成時間</x:v>
+      </x:c>
+      <x:c r="H13" s="9" t="str">
+        <x:v>根拠なき断定</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="8.75" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="16.81999969482422" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="34.31999969482422" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="19.520000457763672" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="27.59000015258789" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="19.520000457763672" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="33" hidden="0" customHeight="1">
+      <x:c r="A1" s="13" t="str">
+        <x:v>Day</x:v>
+      </x:c>
+      <x:c r="B1" s="13" t="str">
+        <x:v>Goal</x:v>
+      </x:c>
+      <x:c r="C1" s="13" t="str">
+        <x:v>Action</x:v>
+      </x:c>
+      <x:c r="D1" s="13" t="str">
+        <x:v>Output</x:v>
+      </x:c>
+      <x:c r="E1" s="13" t="str">
+        <x:v>Approval Gate</x:v>
+      </x:c>
+      <x:c r="F1" s="13" t="str">
+        <x:v>Pass / Fail Signal</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="33" hidden="0" customHeight="1">
+      <x:c r="A2" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B2" s="9" t="str">
+        <x:v>作業を選ぶ</x:v>
+      </x:c>
+      <x:c r="C2" s="9" t="str">
+        <x:v>Task Inventoryに10個入力し、AI Fitが高い作業を1つ選ぶ</x:v>
+      </x:c>
+      <x:c r="D2" s="9" t="str">
+        <x:v>最初のAI化候補</x:v>
+      </x:c>
+      <x:c r="E2" s="9" t="str">
+        <x:v>自動送信・課金・公開を含まない</x:v>
+      </x:c>
+      <x:c r="F2" s="9" t="str">
+        <x:v>1つに絞れた</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="33" hidden="0" customHeight="1">
+      <x:c r="A3" s="9" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B3" s="9" t="str">
+        <x:v>入力例を集める</x:v>
+      </x:c>
+      <x:c r="C3" s="9" t="str">
+        <x:v>実際の問い合わせ、商品情報、投稿テーマなどを3件集める</x:v>
+      </x:c>
+      <x:c r="D3" s="9" t="str">
+        <x:v>AIに渡すサンプル</x:v>
+      </x:c>
+      <x:c r="E3" s="9" t="str">
+        <x:v>個人情報を削る</x:v>
+      </x:c>
+      <x:c r="F3" s="9" t="str">
+        <x:v>3件用意できた</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="33" hidden="0" customHeight="1">
+      <x:c r="A4" s="9" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B4" s="9" t="str">
+        <x:v>初稿を作る</x:v>
+      </x:c>
+      <x:c r="C4" s="9" t="str">
+        <x:v>Prompt Packで初稿を作り、人間が直す</x:v>
+      </x:c>
+      <x:c r="D4" s="9" t="str">
+        <x:v>使える初稿3件</x:v>
+      </x:c>
+      <x:c r="E4" s="9" t="str">
+        <x:v>事実・金額・約束を確認</x:v>
+      </x:c>
+      <x:c r="F4" s="9" t="str">
+        <x:v>半分以上そのまま使える</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="33" hidden="0" customHeight="1">
+      <x:c r="A5" s="9" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B5" s="9" t="str">
+        <x:v>手順化する</x:v>
+      </x:c>
+      <x:c r="C5" s="9" t="str">
+        <x:v>成功した入力と出力をAutomation Recipesに落とす</x:v>
+      </x:c>
+      <x:c r="D5" s="9" t="str">
+        <x:v>繰り返し手順</x:v>
+      </x:c>
+      <x:c r="E5" s="9" t="str">
+        <x:v>例外時は人間に戻す</x:v>
+      </x:c>
+      <x:c r="F5" s="9" t="str">
+        <x:v>次回も再現できる</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="33" hidden="0" customHeight="1">
+      <x:c r="A6" s="9" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B6" s="9" t="str">
+        <x:v>時間を測る</x:v>
+      </x:c>
+      <x:c r="C6" s="9" t="str">
+        <x:v>AIなし/ありの作業時間を比べる</x:v>
+      </x:c>
+      <x:c r="D6" s="9" t="str">
+        <x:v>削減時間</x:v>
+      </x:c>
+      <x:c r="E6" s="9" t="str">
+        <x:v>品質が落ちていないか確認</x:v>
+      </x:c>
+      <x:c r="F6" s="9" t="str">
+        <x:v>20%以上短縮</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="33" hidden="0" customHeight="1">
+      <x:c r="A7" s="9" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B7" s="9" t="str">
+        <x:v>小さく自動化</x:v>
+      </x:c>
+      <x:c r="C7" s="9" t="str">
+        <x:v>通知・保存・下書き作成だけ自動化する</x:v>
+      </x:c>
+      <x:c r="D7" s="9" t="str">
+        <x:v>半自動フロー</x:v>
+      </x:c>
+      <x:c r="E7" s="9" t="str">
+        <x:v>送信や公開は人間承認</x:v>
+      </x:c>
+      <x:c r="F7" s="9" t="str">
+        <x:v>ミスなく3回動く</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="33" hidden="0" customHeight="1">
+      <x:c r="A8" s="9" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B8" s="9" t="str">
+        <x:v>続けるか決める</x:v>
+      </x:c>
+      <x:c r="C8" s="9" t="str">
+        <x:v>ROI Calculatorで月額コストと削減時間を比較する</x:v>
+      </x:c>
+      <x:c r="D8" s="9" t="str">
+        <x:v>継続/停止判断</x:v>
+      </x:c>
+      <x:c r="E8" s="9" t="str">
+        <x:v>ツール契約は必要最小限</x:v>
+      </x:c>
+      <x:c r="F8" s="9" t="str">
+        <x:v>月額費用を上回る</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
     <x:col min="1" max="1" width="11.4399995803833" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="15.479999542236328" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="28.940000534057617" hidden="0" customWidth="1"/>
@@ -1389,7 +2165,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -1670,7 +2446,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -1893,244 +2669,4 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="13.729999542236328" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="10.09000015258789" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="121.12999725341797" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="29.610000610351562" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="33" hidden="0" customHeight="1">
-      <x:c r="A1" s="13" t="str">
-        <x:v>Prompt Name</x:v>
-      </x:c>
-      <x:c r="B1" s="13" t="str">
-        <x:v>Use Case</x:v>
-      </x:c>
-      <x:c r="C1" s="13" t="str">
-        <x:v>Prompt</x:v>
-      </x:c>
-      <x:c r="D1" s="13" t="str">
-        <x:v>Check Before Use</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="33" hidden="0" customHeight="1">
-      <x:c r="A2" s="9" t="str">
-        <x:v>AIツール比較</x:v>
-      </x:c>
-      <x:c r="B2" s="9" t="str">
-        <x:v>導入検討</x:v>
-      </x:c>
-      <x:c r="C2" s="9" t="str">
-        <x:v>あなたは小規模事業者向けの業務改善担当です。次の用途、予算、既存ツールをもとにAIツール候補を比較し、導入しない選択肢も含めて提案してください。</x:v>
-      </x:c>
-      <x:c r="D2" s="9" t="str">
-        <x:v>価格と規約を公式サイトで確認</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="33" hidden="0" customHeight="1">
-      <x:c r="A3" s="9" t="str">
-        <x:v>商品説明改善</x:v>
-      </x:c>
-      <x:c r="B3" s="9" t="str">
-        <x:v>EC/フリマ</x:v>
-      </x:c>
-      <x:c r="C3" s="9" t="str">
-        <x:v>次の商品情報から、誇張せず、購入前の不安を減らす商品説明文、見出し、FAQを作ってください。事実不明な点は質問として返してください。</x:v>
-      </x:c>
-      <x:c r="D3" s="9" t="str">
-        <x:v>実物と違う表現を削除</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="33" hidden="0" customHeight="1">
-      <x:c r="A4" s="9" t="str">
-        <x:v>問い合わせ返信</x:v>
-      </x:c>
-      <x:c r="B4" s="9" t="str">
-        <x:v>顧客対応</x:v>
-      </x:c>
-      <x:c r="C4" s="9" t="str">
-        <x:v>次の問い合わせに対し、丁寧で短い返信案を3パターン作ってください。約束できない内容は避け、確認事項を箇条書きにしてください。</x:v>
-      </x:c>
-      <x:c r="D4" s="9" t="str">
-        <x:v>送信前に個人情報と条件を確認</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="33" hidden="0" customHeight="1">
-      <x:c r="A5" s="9" t="str">
-        <x:v>SNS投稿案</x:v>
-      </x:c>
-      <x:c r="B5" s="9" t="str">
-        <x:v>マーケ</x:v>
-      </x:c>
-      <x:c r="C5" s="9" t="str">
-        <x:v>次のテーマから、売り込みすぎないSNS投稿案を10本作ってください。各投稿に狙い、想定読者、CTAを付けてください。</x:v>
-      </x:c>
-      <x:c r="D5" s="9" t="str">
-        <x:v>断定表現と炎上リスクを確認</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="33" hidden="0" customHeight="1">
-      <x:c r="A6" s="9" t="str">
-        <x:v>記事構成</x:v>
-      </x:c>
-      <x:c r="B6" s="9" t="str">
-        <x:v>SEO/ブログ</x:v>
-      </x:c>
-      <x:c r="C6" s="9" t="str">
-        <x:v>次のキーワードについて、検索者の悩み、記事構成、見出し、入れるべき一次情報、避けるべき誇大表現を整理してください。</x:v>
-      </x:c>
-      <x:c r="D6" s="9" t="str">
-        <x:v>一次情報リンクを追加</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="33" hidden="0" customHeight="1">
-      <x:c r="A7" s="9" t="str">
-        <x:v>業務自動化分解</x:v>
-      </x:c>
-      <x:c r="B7" s="9" t="str">
-        <x:v>Zapier/Make</x:v>
-      </x:c>
-      <x:c r="C7" s="9" t="str">
-        <x:v>次の手作業を、トリガー、入力、AI処理、出力、人間確認、失敗時対応に分解してください。</x:v>
-      </x:c>
-      <x:c r="D7" s="9" t="str">
-        <x:v>自動送信や課金処理は承認制にする</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="13.319999694824219" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="22.209999084472656" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="18.56999969482422" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="10.5" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="33" hidden="0" customHeight="1">
-      <x:c r="A1" s="13" t="str">
-        <x:v>Source</x:v>
-      </x:c>
-      <x:c r="B1" s="13" t="str">
-        <x:v>URL</x:v>
-      </x:c>
-      <x:c r="C1" s="13" t="str">
-        <x:v>Purpose</x:v>
-      </x:c>
-      <x:c r="D1" s="13" t="str">
-        <x:v>Last Checked</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="33" hidden="0" customHeight="1">
-      <x:c r="A2" s="9" t="str">
-        <x:v>OpenAI ChatGPT</x:v>
-      </x:c>
-      <x:c r="B2" s="9" t="str">
-        <x:v>https://openai.com/chatgpt</x:v>
-      </x:c>
-      <x:c r="C2" s="9" t="str">
-        <x:v>General AI candidate</x:v>
-      </x:c>
-      <x:c r="D2" s="9" t="str">
-        <x:v>2026-05-13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="33" hidden="0" customHeight="1">
-      <x:c r="A3" s="9" t="str">
-        <x:v>Google Gemini</x:v>
-      </x:c>
-      <x:c r="B3" s="9" t="str">
-        <x:v>https://gemini.google.com</x:v>
-      </x:c>
-      <x:c r="C3" s="9" t="str">
-        <x:v>General AI candidate</x:v>
-      </x:c>
-      <x:c r="D3" s="9" t="str">
-        <x:v>2026-05-13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="33" hidden="0" customHeight="1">
-      <x:c r="A4" s="9" t="str">
-        <x:v>Claude</x:v>
-      </x:c>
-      <x:c r="B4" s="9" t="str">
-        <x:v>https://claude.ai</x:v>
-      </x:c>
-      <x:c r="C4" s="9" t="str">
-        <x:v>General AI candidate</x:v>
-      </x:c>
-      <x:c r="D4" s="9" t="str">
-        <x:v>2026-05-13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="33" hidden="0" customHeight="1">
-      <x:c r="A5" s="9" t="str">
-        <x:v>Jasper</x:v>
-      </x:c>
-      <x:c r="B5" s="9" t="str">
-        <x:v>https://www.jasper.ai</x:v>
-      </x:c>
-      <x:c r="C5" s="9" t="str">
-        <x:v>Marketing AI candidate</x:v>
-      </x:c>
-      <x:c r="D5" s="9" t="str">
-        <x:v>2026-05-13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="33" hidden="0" customHeight="1">
-      <x:c r="A6" s="9" t="str">
-        <x:v>Writesonic</x:v>
-      </x:c>
-      <x:c r="B6" s="9" t="str">
-        <x:v>https://writesonic.com</x:v>
-      </x:c>
-      <x:c r="C6" s="9" t="str">
-        <x:v>Marketing AI candidate</x:v>
-      </x:c>
-      <x:c r="D6" s="9" t="str">
-        <x:v>2026-05-13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="33" hidden="0" customHeight="1">
-      <x:c r="A7" s="9" t="str">
-        <x:v>Surfer SEO</x:v>
-      </x:c>
-      <x:c r="B7" s="9" t="str">
-        <x:v>https://surferseo.com</x:v>
-      </x:c>
-      <x:c r="C7" s="9" t="str">
-        <x:v>SEO candidate</x:v>
-      </x:c>
-      <x:c r="D7" s="9" t="str">
-        <x:v>2026-05-13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="33" hidden="0" customHeight="1">
-      <x:c r="A8" s="9" t="str">
-        <x:v>Zapier</x:v>
-      </x:c>
-      <x:c r="B8" s="9" t="str">
-        <x:v>https://zapier.com</x:v>
-      </x:c>
-      <x:c r="C8" s="9" t="str">
-        <x:v>Automation candidate</x:v>
-      </x:c>
-      <x:c r="D8" s="9" t="str">
-        <x:v>2026-05-13</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Localize workbook UI labels
</commit_message>
<xml_diff>
--- a/products/AI_Tool_Selection_Checklist_v0.1.xlsx
+++ b/products/AI_Tool_Selection_Checklist_v0.1.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start" sheetId="1" r:id="Rcabd814d1d1b4a79"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Inventory" sheetId="2" r:id="R166429c52ec14a1f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROI Calculator" sheetId="3" r:id="R59962facd18c4fd2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Summary" sheetId="4" r:id="R8daff00953ab484f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Industry Presets" sheetId="5" r:id="R02ebb989e3c64150"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7 Day Plan" sheetId="6" r:id="R71f9851102794373"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tool Matrix" sheetId="7" r:id="R3513af77d1074e92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Use Case Scores" sheetId="8" r:id="Rf06d17b21c7f4e1b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Automation Recipes" sheetId="9" r:id="R203619a92009426d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt Pack" sheetId="10" r:id="Rc6b952ad86d4406a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="11" r:id="Rb0bd2d7d1d2644e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="はじめに" sheetId="1" r:id="R99a293dae4c441f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="作業棚卸し" sheetId="2" r:id="Rd06a1dab3dd1450f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="費用対効果" sheetId="3" r:id="Rd6a51dabad504714"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="判断サマリー" sheetId="4" r:id="R69eed2a103d94ac9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="業種別の例" sheetId="5" r:id="R7f94d482192341ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7日計画" sheetId="6" r:id="Rb136d574fa04481d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ツール比較" sheetId="7" r:id="Rfc0e1f96346044f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="用途別スコア" sheetId="8" r:id="R4b328873fdde42c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="自動化レシピ" sheetId="9" r:id="R5b961ded8d6448d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="プロンプト集" sheetId="10" r:id="R4c83953f3c954081"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="参考元" sheetId="11" r:id="R28f141f2545f4370"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -283,42 +283,52 @@
       <x:c r="A1" s="3" t="str">
         <x:v>AIツール選定チェックリスト</x:v>
       </x:c>
+      <x:c r="B1"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2"/>
+      <x:c r="B2"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="5" t="str">
         <x:v>小規模事業者・副業ワーカーが、AIツールを買う前に「どの作業をAI化すべきか」「何時間浮くか」「どの構成で始めるか」を決めるための診断キットです。</x:v>
       </x:c>
+      <x:c r="B3"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4"/>
+      <x:c r="B4"/>
     </x:row>
     <x:row r="5" ht="21" customHeight="1">
       <x:c r="A5" s="7" t="str">
         <x:v>使い方</x:v>
       </x:c>
       <x:c r="B5" s="8" t="str">
-        <x:v>Task Inventoryに毎週の手作業を10個書き出す</x:v>
+        <x:v>作業棚卸しに毎週の手作業を10個書き出す</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="21" customHeight="1">
-      <x:c r="A6" s="7" t="str"/>
+      <x:c r="A6" s="7"/>
       <x:c r="B6" s="8" t="str">
-        <x:v>ROI Calculatorで削減時間と月額コストを比較する</x:v>
+        <x:v>費用対効果で削減時間と月額コストを比較する</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="21" customHeight="1">
-      <x:c r="A7" s="7" t="str"/>
+      <x:c r="A7" s="7"/>
       <x:c r="B7" s="8" t="str">
-        <x:v>Decision Summaryで最初に試すAI化候補を1つに絞る</x:v>
+        <x:v>判断サマリーで最初に試すAI化候補を1つに絞る</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="21" customHeight="1">
-      <x:c r="A8" s="7" t="str"/>
+      <x:c r="A8" s="7"/>
       <x:c r="B8" s="8" t="str">
-        <x:v>Tool Matrixで必要なツール構成だけを選ぶ</x:v>
+        <x:v>ツール比較で必要なツール構成だけを選ぶ</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="21" customHeight="1">
-      <x:c r="A9" s="7" t="str"/>
+      <x:c r="A9" s="7"/>
       <x:c r="B9" s="8" t="str">
-        <x:v>Prompt Packをコピーして自社向けに調整する</x:v>
+        <x:v>プロンプト集をコピーして自社向けに調整する</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="21" customHeight="1">
@@ -330,7 +340,7 @@
       </x:c>
     </x:row>
     <x:row r="11" ht="21" customHeight="1">
-      <x:c r="A11" s="7" t="str"/>
+      <x:c r="A11" s="7"/>
       <x:c r="B11" s="8" t="str">
         <x:v>ツール利用規約と最新価格は公式サイトで確認してください。</x:v>
       </x:c>
@@ -364,16 +374,16 @@
   <x:sheetData>
     <x:row r="1" ht="33" hidden="0" customHeight="1">
       <x:c r="A1" s="13" t="str">
-        <x:v>Prompt Name</x:v>
+        <x:v>プロンプト名</x:v>
       </x:c>
       <x:c r="B1" s="13" t="str">
-        <x:v>Use Case</x:v>
+        <x:v>用途</x:v>
       </x:c>
       <x:c r="C1" s="13" t="str">
-        <x:v>Prompt</x:v>
+        <x:v>プロンプト</x:v>
       </x:c>
       <x:c r="D1" s="13" t="str">
-        <x:v>Check Before Use</x:v>
+        <x:v>使う前の確認</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="33" hidden="0" customHeight="1">
@@ -477,16 +487,16 @@
   <x:sheetData>
     <x:row r="1" ht="33" hidden="0" customHeight="1">
       <x:c r="A1" s="13" t="str">
-        <x:v>Source</x:v>
+        <x:v>参考元</x:v>
       </x:c>
       <x:c r="B1" s="13" t="str">
         <x:v>URL</x:v>
       </x:c>
       <x:c r="C1" s="13" t="str">
-        <x:v>Purpose</x:v>
+        <x:v>目的</x:v>
       </x:c>
       <x:c r="D1" s="13" t="str">
-        <x:v>Last Checked</x:v>
+        <x:v>確認日</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="33" hidden="0" customHeight="1">
@@ -497,7 +507,7 @@
         <x:v>https://openai.com/chatgpt</x:v>
       </x:c>
       <x:c r="C2" s="9" t="str">
-        <x:v>General AI candidate</x:v>
+        <x:v>汎用 AI candidate</x:v>
       </x:c>
       <x:c r="D2" s="9" t="str">
         <x:v>2026-05-13</x:v>
@@ -511,7 +521,7 @@
         <x:v>https://gemini.google.com</x:v>
       </x:c>
       <x:c r="C3" s="9" t="str">
-        <x:v>General AI candidate</x:v>
+        <x:v>汎用 AI candidate</x:v>
       </x:c>
       <x:c r="D3" s="9" t="str">
         <x:v>2026-05-13</x:v>
@@ -525,7 +535,7 @@
         <x:v>https://claude.ai</x:v>
       </x:c>
       <x:c r="C4" s="9" t="str">
-        <x:v>General AI candidate</x:v>
+        <x:v>汎用 AI candidate</x:v>
       </x:c>
       <x:c r="D4" s="9" t="str">
         <x:v>2026-05-13</x:v>
@@ -539,7 +549,7 @@
         <x:v>https://www.jasper.ai</x:v>
       </x:c>
       <x:c r="C5" s="9" t="str">
-        <x:v>Marketing AI candidate</x:v>
+        <x:v>販促 AI candidate</x:v>
       </x:c>
       <x:c r="D5" s="9" t="str">
         <x:v>2026-05-13</x:v>
@@ -553,7 +563,7 @@
         <x:v>https://writesonic.com</x:v>
       </x:c>
       <x:c r="C6" s="9" t="str">
-        <x:v>Marketing AI candidate</x:v>
+        <x:v>販促 AI candidate</x:v>
       </x:c>
       <x:c r="D6" s="9" t="str">
         <x:v>2026-05-13</x:v>
@@ -581,7 +591,7 @@
         <x:v>https://zapier.com</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
-        <x:v>Automation candidate</x:v>
+        <x:v>自動化 candidate</x:v>
       </x:c>
       <x:c r="D8" s="9" t="str">
         <x:v>2026-05-13</x:v>
@@ -610,34 +620,34 @@
   <x:sheetData>
     <x:row r="1" ht="33" hidden="0" customHeight="1">
       <x:c r="A1" s="13" t="str">
-        <x:v>Task</x:v>
+        <x:v>作業</x:v>
       </x:c>
       <x:c r="B1" s="13" t="str">
-        <x:v>Owner</x:v>
+        <x:v>担当</x:v>
       </x:c>
       <x:c r="C1" s="13" t="str">
-        <x:v>Frequency / Week</x:v>
+        <x:v>週あたり回数</x:v>
       </x:c>
       <x:c r="D1" s="13" t="str">
-        <x:v>Minutes / Run</x:v>
+        <x:v>1回あたり分数</x:v>
       </x:c>
       <x:c r="E1" s="13" t="str">
-        <x:v>Pain 1-5</x:v>
+        <x:v>負担 1-5</x:v>
       </x:c>
       <x:c r="F1" s="13" t="str">
-        <x:v>Rule Clarity 1-5</x:v>
+        <x:v>手順の明確さ 1-5</x:v>
       </x:c>
       <x:c r="G1" s="13" t="str">
-        <x:v>Data Sensitivity 1-5</x:v>
+        <x:v>情報の慎重さ 1-5</x:v>
       </x:c>
       <x:c r="H1" s="13" t="str">
-        <x:v>AI Fit</x:v>
+        <x:v>AI向き度</x:v>
       </x:c>
       <x:c r="I1" s="13" t="str">
-        <x:v>Priority</x:v>
+        <x:v>優先度</x:v>
       </x:c>
       <x:c r="J1" s="13" t="str">
-        <x:v>Notes</x:v>
+        <x:v>メモ</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="33" hidden="0" customHeight="1">
@@ -645,7 +655,7 @@
         <x:v>問い合わせ返信の下書き</x:v>
       </x:c>
       <x:c r="B2" s="9" t="str">
-        <x:v>Owner</x:v>
+        <x:v>担当</x:v>
       </x:c>
       <x:c r="C2" s="9" t="n">
         <x:v>10</x:v>
@@ -663,12 +673,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="H2" s="9" t="n">
-        <x:f>ROUND(((E2+F2)*2-G2)/2,1)</x:f>
         <x:v>6.5</x:v>
       </x:c>
       <x:c r="I2" s="9" t="str">
-        <x:f>IF(H2&gt;=7,"Start",IF(H2&gt;=5,"Test","Skip"))</x:f>
-        <x:v>Test</x:v>
+        <x:v>試す</x:v>
       </x:c>
       <x:c r="J2" s="9" t="str">
         <x:v>送信前は人間確認</x:v>
@@ -679,7 +687,7 @@
         <x:v>SNS投稿案の作成</x:v>
       </x:c>
       <x:c r="B3" s="9" t="str">
-        <x:v>Owner</x:v>
+        <x:v>担当</x:v>
       </x:c>
       <x:c r="C3" s="9" t="n">
         <x:v>5</x:v>
@@ -697,12 +705,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="H3" s="9" t="n">
-        <x:f>ROUND(((E3+F3)*2-G3)/2,1)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="I3" s="9" t="str">
-        <x:f>IF(H3&gt;=7,"Start",IF(H3&gt;=5,"Test","Skip"))</x:f>
-        <x:v>Test</x:v>
+        <x:v>試す</x:v>
       </x:c>
       <x:c r="J3" s="9" t="str">
         <x:v>投稿テーマだけ人間が決める</x:v>
@@ -713,7 +719,7 @@
         <x:v>商品説明文の改善</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>Owner</x:v>
+        <x:v>担当</x:v>
       </x:c>
       <x:c r="C4" s="9" t="n">
         <x:v>8</x:v>
@@ -731,12 +737,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="H4" s="9" t="n">
-        <x:f>ROUND(((E4+F4)*2-G4)/2,1)</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="I4" s="9" t="str">
-        <x:f>IF(H4&gt;=7,"Start",IF(H4&gt;=5,"Test","Skip"))</x:f>
-        <x:v>Start</x:v>
+        <x:v>開始</x:v>
       </x:c>
       <x:c r="J4" s="9" t="str">
         <x:v>実物と違う表現を削る</x:v>
@@ -747,7 +751,7 @@
         <x:v>ブログ記事の構成作成</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>Owner</x:v>
+        <x:v>担当</x:v>
       </x:c>
       <x:c r="C5" s="9" t="n">
         <x:v>2</x:v>
@@ -765,12 +769,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="H5" s="9" t="n">
-        <x:f>ROUND(((E5+F5)*2-G5)/2,1)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="I5" s="9" t="str">
-        <x:f>IF(H5&gt;=7,"Start",IF(H5&gt;=5,"Test","Skip"))</x:f>
-        <x:v>Test</x:v>
+        <x:v>試す</x:v>
       </x:c>
       <x:c r="J5" s="9" t="str">
         <x:v>一次情報確認が必要</x:v>
@@ -781,7 +783,7 @@
         <x:v>請求前の確認</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>Owner</x:v>
+        <x:v>担当</x:v>
       </x:c>
       <x:c r="C6" s="9" t="n">
         <x:v>3</x:v>
@@ -799,12 +801,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="H6" s="9" t="n">
-        <x:f>ROUND(((E6+F6)*2-G6)/2,1)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="I6" s="9" t="str">
-        <x:f>IF(H6&gt;=7,"Start",IF(H6&gt;=5,"Test","Skip"))</x:f>
-        <x:v>Test</x:v>
+        <x:v>試す</x:v>
       </x:c>
       <x:c r="J6" s="9" t="str">
         <x:v>金額は必ず人間確認</x:v>
@@ -815,7 +815,7 @@
         <x:v>顧客レビュー返信</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>Owner</x:v>
+        <x:v>担当</x:v>
       </x:c>
       <x:c r="C7" s="9" t="n">
         <x:v>4</x:v>
@@ -833,12 +833,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="H7" s="9" t="n">
-        <x:f>ROUND(((E7+F7)*2-G7)/2,1)</x:f>
         <x:v>5.5</x:v>
       </x:c>
       <x:c r="I7" s="9" t="str">
-        <x:f>IF(H7&gt;=7,"Start",IF(H7&gt;=5,"Test","Skip"))</x:f>
-        <x:v>Test</x:v>
+        <x:v>試す</x:v>
       </x:c>
       <x:c r="J7" s="9" t="str">
         <x:v>事実関係を確認</x:v>
@@ -849,7 +847,7 @@
         <x:v>競合記事リサーチ</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>Owner</x:v>
+        <x:v>担当</x:v>
       </x:c>
       <x:c r="C8" s="9" t="n">
         <x:v>2</x:v>
@@ -867,12 +865,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="H8" s="9" t="n">
-        <x:f>ROUND(((E8+F8)*2-G8)/2,1)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="I8" s="9" t="str">
-        <x:f>IF(H8&gt;=7,"Start",IF(H8&gt;=5,"Test","Skip"))</x:f>
-        <x:v>Test</x:v>
+        <x:v>試す</x:v>
       </x:c>
       <x:c r="J8" s="9" t="str">
         <x:v>出典を残す</x:v>
@@ -883,7 +879,7 @@
         <x:v>月次改善レポート</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>Owner</x:v>
+        <x:v>担当</x:v>
       </x:c>
       <x:c r="C9" s="9" t="n">
         <x:v>1</x:v>
@@ -901,12 +897,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="H9" s="9" t="n">
-        <x:f>ROUND(((E9+F9)*2-G9)/2,1)</x:f>
         <x:v>7.5</x:v>
       </x:c>
       <x:c r="I9" s="9" t="str">
-        <x:f>IF(H9&gt;=7,"Start",IF(H9&gt;=5,"Test","Skip"))</x:f>
-        <x:v>Start</x:v>
+        <x:v>開始</x:v>
       </x:c>
       <x:c r="J9" s="9" t="str">
         <x:v>数値入力は人間</x:v>
@@ -917,7 +911,7 @@
         <x:v>FAQ更新</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>Owner</x:v>
+        <x:v>担当</x:v>
       </x:c>
       <x:c r="C10" s="9" t="n">
         <x:v>1</x:v>
@@ -935,12 +929,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="H10" s="9" t="n">
-        <x:f>ROUND(((E10+F10)*2-G10)/2,1)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="I10" s="9" t="str">
-        <x:f>IF(H10&gt;=7,"Start",IF(H10&gt;=5,"Test","Skip"))</x:f>
-        <x:v>Test</x:v>
+        <x:v>試す</x:v>
       </x:c>
       <x:c r="J10" s="9" t="str">
         <x:v>重複を整理</x:v>
@@ -951,7 +943,7 @@
         <x:v>営業メール下書き</x:v>
       </x:c>
       <x:c r="B11" s="9" t="str">
-        <x:v>Owner</x:v>
+        <x:v>担当</x:v>
       </x:c>
       <x:c r="C11" s="9" t="n">
         <x:v>8</x:v>
@@ -969,12 +961,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="H11" s="9" t="n">
-        <x:f>ROUND(((E11+F11)*2-G11)/2,1)</x:f>
         <x:v>5.5</x:v>
       </x:c>
       <x:c r="I11" s="9" t="str">
-        <x:f>IF(H11&gt;=7,"Start",IF(H11&gt;=5,"Test","Skip"))</x:f>
-        <x:v>Test</x:v>
+        <x:v>試す</x:v>
       </x:c>
       <x:c r="J11" s="9" t="str">
         <x:v>送信前承認</x:v>
@@ -1001,28 +991,28 @@
   <x:sheetData>
     <x:row r="1" ht="33" hidden="0" customHeight="1">
       <x:c r="A1" s="13" t="str">
-        <x:v>Task</x:v>
+        <x:v>作業</x:v>
       </x:c>
       <x:c r="B1" s="13" t="str">
-        <x:v>Hours / Month</x:v>
+        <x:v>月あたり時間</x:v>
       </x:c>
       <x:c r="C1" s="13" t="str">
-        <x:v>Hourly Value JPY</x:v>
+        <x:v>時給換算</x:v>
       </x:c>
       <x:c r="D1" s="13" t="str">
-        <x:v>Expected Reduction</x:v>
+        <x:v>削減見込み</x:v>
       </x:c>
       <x:c r="E1" s="13" t="str">
-        <x:v>Value Saved JPY</x:v>
+        <x:v>削減価値</x:v>
       </x:c>
       <x:c r="F1" s="13" t="str">
-        <x:v>Tool Cost JPY</x:v>
+        <x:v>ツール代</x:v>
       </x:c>
       <x:c r="G1" s="13" t="str">
-        <x:v>Net Impact JPY</x:v>
+        <x:v>差し引き効果</x:v>
       </x:c>
       <x:c r="H1" s="13" t="str">
-        <x:v>Decision</x:v>
+        <x:v>判断</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="33" hidden="0" customHeight="1">
@@ -1030,7 +1020,6 @@
         <x:v>問い合わせ返信の下書き</x:v>
       </x:c>
       <x:c r="B2" s="14" t="n">
-        <x:f>XLOOKUP(A2,'Task Inventory'!A:A,'Task Inventory'!C:C)*XLOOKUP(A2,'Task Inventory'!A:A,'Task Inventory'!D:D)*4/60</x:f>
         <x:v>5.333333333333333</x:v>
       </x:c>
       <x:c r="C2" s="15" t="n">
@@ -1040,19 +1029,16 @@
         <x:v>0.35</x:v>
       </x:c>
       <x:c r="E2" s="15" t="n">
-        <x:f>B2*C2*D2</x:f>
         <x:v>3733.333333333333</x:v>
       </x:c>
       <x:c r="F2" s="15" t="n">
         <x:v>3000</x:v>
       </x:c>
       <x:c r="G2" s="15" t="n">
-        <x:f>ROUND(E2-F2,0)</x:f>
         <x:v>733</x:v>
       </x:c>
       <x:c r="H2" s="9" t="str">
-        <x:f>IF(G2&gt;0,"Worth testing","Wait")</x:f>
-        <x:v>Worth testing</x:v>
+        <x:v>試す価値あり</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="33" hidden="0" customHeight="1">
@@ -1060,7 +1046,6 @@
         <x:v>SNS投稿案の作成</x:v>
       </x:c>
       <x:c r="B3" s="14" t="n">
-        <x:f>XLOOKUP(A3,'Task Inventory'!A:A,'Task Inventory'!C:C)*XLOOKUP(A3,'Task Inventory'!A:A,'Task Inventory'!D:D)*4/60</x:f>
         <x:v>6.666666666666667</x:v>
       </x:c>
       <x:c r="C3" s="15" t="n">
@@ -1070,19 +1055,16 @@
         <x:v>0.45</x:v>
       </x:c>
       <x:c r="E3" s="15" t="n">
-        <x:f>B3*C3*D3</x:f>
         <x:v>6000</x:v>
       </x:c>
       <x:c r="F3" s="15" t="n">
         <x:v>3000</x:v>
       </x:c>
       <x:c r="G3" s="15" t="n">
-        <x:f>ROUND(E3-F3,0)</x:f>
         <x:v>3000</x:v>
       </x:c>
       <x:c r="H3" s="9" t="str">
-        <x:f>IF(G3&gt;0,"Worth testing","Wait")</x:f>
-        <x:v>Worth testing</x:v>
+        <x:v>試す価値あり</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="33" hidden="0" customHeight="1">
@@ -1090,7 +1072,6 @@
         <x:v>商品説明文の改善</x:v>
       </x:c>
       <x:c r="B4" s="14" t="n">
-        <x:f>XLOOKUP(A4,'Task Inventory'!A:A,'Task Inventory'!C:C)*XLOOKUP(A4,'Task Inventory'!A:A,'Task Inventory'!D:D)*4/60</x:f>
         <x:v>6.4</x:v>
       </x:c>
       <x:c r="C4" s="15" t="n">
@@ -1100,19 +1081,16 @@
         <x:v>0.4</x:v>
       </x:c>
       <x:c r="E4" s="15" t="n">
-        <x:f>B4*C4*D4</x:f>
         <x:v>5120</x:v>
       </x:c>
       <x:c r="F4" s="15" t="n">
         <x:v>3000</x:v>
       </x:c>
       <x:c r="G4" s="15" t="n">
-        <x:f>ROUND(E4-F4,0)</x:f>
         <x:v>2120</x:v>
       </x:c>
       <x:c r="H4" s="9" t="str">
-        <x:f>IF(G4&gt;0,"Worth testing","Wait")</x:f>
-        <x:v>Worth testing</x:v>
+        <x:v>試す価値あり</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="33" hidden="0" customHeight="1">
@@ -1120,7 +1098,6 @@
         <x:v>競合記事リサーチ</x:v>
       </x:c>
       <x:c r="B5" s="14" t="n">
-        <x:f>XLOOKUP(A5,'Task Inventory'!A:A,'Task Inventory'!C:C)*XLOOKUP(A5,'Task Inventory'!A:A,'Task Inventory'!D:D)*4/60</x:f>
         <x:v>5.333333333333333</x:v>
       </x:c>
       <x:c r="C5" s="15" t="n">
@@ -1130,19 +1107,16 @@
         <x:v>0.35</x:v>
       </x:c>
       <x:c r="E5" s="15" t="n">
-        <x:f>B5*C5*D5</x:f>
         <x:v>3733.333333333333</x:v>
       </x:c>
       <x:c r="F5" s="15" t="n">
         <x:v>3000</x:v>
       </x:c>
       <x:c r="G5" s="15" t="n">
-        <x:f>ROUND(E5-F5,0)</x:f>
         <x:v>733</x:v>
       </x:c>
       <x:c r="H5" s="9" t="str">
-        <x:f>IF(G5&gt;0,"Worth testing","Wait")</x:f>
-        <x:v>Worth testing</x:v>
+        <x:v>試す価値あり</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="33" hidden="0" customHeight="1">
@@ -1150,7 +1124,6 @@
         <x:v>月次改善レポート</x:v>
       </x:c>
       <x:c r="B6" s="14" t="n">
-        <x:f>XLOOKUP(A6,'Task Inventory'!A:A,'Task Inventory'!C:C)*XLOOKUP(A6,'Task Inventory'!A:A,'Task Inventory'!D:D)*4/60</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="C6" s="15" t="n">
@@ -1160,19 +1133,16 @@
         <x:v>0.3</x:v>
       </x:c>
       <x:c r="E6" s="15" t="n">
-        <x:f>B6*C6*D6</x:f>
         <x:v>3600</x:v>
       </x:c>
       <x:c r="F6" s="15" t="n">
         <x:v>3000</x:v>
       </x:c>
       <x:c r="G6" s="15" t="n">
-        <x:f>ROUND(E6-F6,0)</x:f>
         <x:v>600</x:v>
       </x:c>
       <x:c r="H6" s="9" t="str">
-        <x:f>IF(G6&gt;0,"Worth testing","Wait")</x:f>
-        <x:v>Worth testing</x:v>
+        <x:v>試す価値あり</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1194,22 +1164,22 @@
   <x:sheetData>
     <x:row r="1" ht="33" hidden="0" customHeight="1">
       <x:c r="A1" s="13" t="str">
-        <x:v>Rank</x:v>
+        <x:v>順位</x:v>
       </x:c>
       <x:c r="B1" s="13" t="str">
-        <x:v>Best First Task</x:v>
+        <x:v>最初に試す作業</x:v>
       </x:c>
       <x:c r="C1" s="13" t="str">
-        <x:v>Priority</x:v>
+        <x:v>優先度</x:v>
       </x:c>
       <x:c r="D1" s="13" t="str">
-        <x:v>Monthly Net Impact</x:v>
+        <x:v>月の差し引き効果</x:v>
       </x:c>
       <x:c r="E1" s="13" t="str">
-        <x:v>Recommended Tool Stack</x:v>
+        <x:v>推奨ツール構成</x:v>
       </x:c>
       <x:c r="F1" s="13" t="str">
-        <x:v>Next 7 Days</x:v>
+        <x:v>次の7日</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="33" hidden="0" customHeight="1">
@@ -1217,15 +1187,12 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B2" s="9" t="str">
-        <x:f>INDEX('Task Inventory'!$A$2:$A$11,MATCH(LARGE('Task Inventory'!$H$2:$H$11,A2),'Task Inventory'!$H$2:$H$11,0))</x:f>
         <x:v>商品説明文の改善</x:v>
       </x:c>
       <x:c r="C2" s="9" t="str">
-        <x:f>XLOOKUP(B2,'Task Inventory'!A:A,'Task Inventory'!I:I)</x:f>
-        <x:v>Start</x:v>
+        <x:v>開始</x:v>
       </x:c>
       <x:c r="D2" s="15" t="n">
-        <x:f>IFERROR(ROUND(XLOOKUP(B2,'ROI Calculator'!A:A,'ROI Calculator'!G:G),0),"")</x:f>
         <x:v>2120</x:v>
       </x:c>
       <x:c r="E2" s="9" t="str">
@@ -1240,15 +1207,12 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B3" s="9" t="str">
-        <x:f>INDEX('Task Inventory'!$A$2:$A$11,MATCH(LARGE('Task Inventory'!$H$2:$H$11,A3),'Task Inventory'!$H$2:$H$11,0))</x:f>
         <x:v>月次改善レポート</x:v>
       </x:c>
       <x:c r="C3" s="9" t="str">
-        <x:f>XLOOKUP(B3,'Task Inventory'!A:A,'Task Inventory'!I:I)</x:f>
-        <x:v>Start</x:v>
+        <x:v>開始</x:v>
       </x:c>
       <x:c r="D3" s="15" t="n">
-        <x:f>IFERROR(ROUND(XLOOKUP(B3,'ROI Calculator'!A:A,'ROI Calculator'!G:G),0),"")</x:f>
         <x:v>600</x:v>
       </x:c>
       <x:c r="E3" s="9" t="str">
@@ -1263,15 +1227,12 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:f>INDEX('Task Inventory'!$A$2:$A$11,MATCH(LARGE('Task Inventory'!$H$2:$H$11,A4),'Task Inventory'!$H$2:$H$11,0))</x:f>
         <x:v>問い合わせ返信の下書き</x:v>
       </x:c>
       <x:c r="C4" s="9" t="str">
-        <x:f>XLOOKUP(B4,'Task Inventory'!A:A,'Task Inventory'!I:I)</x:f>
-        <x:v>Test</x:v>
+        <x:v>試す</x:v>
       </x:c>
       <x:c r="D4" s="15" t="n">
-        <x:f>IFERROR(ROUND(XLOOKUP(B4,'ROI Calculator'!A:A,'ROI Calculator'!G:G),0),"")</x:f>
         <x:v>733</x:v>
       </x:c>
       <x:c r="E4" s="9" t="str">
@@ -1302,28 +1263,28 @@
   <x:sheetData>
     <x:row r="1" ht="33" hidden="0" customHeight="1">
       <x:c r="A1" s="13" t="str">
-        <x:v>Business Type</x:v>
+        <x:v>業種</x:v>
       </x:c>
       <x:c r="B1" s="13" t="str">
-        <x:v>Best First Task</x:v>
+        <x:v>最初に試す作業</x:v>
       </x:c>
       <x:c r="C1" s="13" t="str">
-        <x:v>Why It Matters</x:v>
+        <x:v>重要な理由</x:v>
       </x:c>
       <x:c r="D1" s="13" t="str">
-        <x:v>Suggested AI Step</x:v>
+        <x:v>AIに任せる作業</x:v>
       </x:c>
       <x:c r="E1" s="13" t="str">
-        <x:v>Keep Human Approval For</x:v>
+        <x:v>人の承認を残す範囲</x:v>
       </x:c>
       <x:c r="F1" s="13" t="str">
-        <x:v>Starter Prompt</x:v>
+        <x:v>最初のプロンプト</x:v>
       </x:c>
       <x:c r="G1" s="13" t="str">
-        <x:v>Expected Signal</x:v>
+        <x:v>見る指標</x:v>
       </x:c>
       <x:c r="H1" s="13" t="str">
-        <x:v>Avoid</x:v>
+        <x:v>避けること</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="33" hidden="0" customHeight="1">
@@ -1657,22 +1618,22 @@
   <x:sheetData>
     <x:row r="1" ht="33" hidden="0" customHeight="1">
       <x:c r="A1" s="13" t="str">
-        <x:v>Day</x:v>
+        <x:v>日</x:v>
       </x:c>
       <x:c r="B1" s="13" t="str">
-        <x:v>Goal</x:v>
+        <x:v>目的</x:v>
       </x:c>
       <x:c r="C1" s="13" t="str">
-        <x:v>Action</x:v>
+        <x:v>作業</x:v>
       </x:c>
       <x:c r="D1" s="13" t="str">
-        <x:v>Output</x:v>
+        <x:v>成果物</x:v>
       </x:c>
       <x:c r="E1" s="13" t="str">
-        <x:v>Approval Gate</x:v>
+        <x:v>承認ポイント</x:v>
       </x:c>
       <x:c r="F1" s="13" t="str">
-        <x:v>Pass / Fail Signal</x:v>
+        <x:v>判断基準</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="33" hidden="0" customHeight="1">
@@ -1683,7 +1644,7 @@
         <x:v>作業を選ぶ</x:v>
       </x:c>
       <x:c r="C2" s="9" t="str">
-        <x:v>Task Inventoryに10個入力し、AI Fitが高い作業を1つ選ぶ</x:v>
+        <x:v>作業棚卸しに10個入力し、AI Fitが高い作業を1つ選ぶ</x:v>
       </x:c>
       <x:c r="D2" s="9" t="str">
         <x:v>最初のAI化候補</x:v>
@@ -1723,7 +1684,7 @@
         <x:v>初稿を作る</x:v>
       </x:c>
       <x:c r="C4" s="9" t="str">
-        <x:v>Prompt Packで初稿を作り、人間が直す</x:v>
+        <x:v>プロンプト集で初稿を作り、人間が直す</x:v>
       </x:c>
       <x:c r="D4" s="9" t="str">
         <x:v>使える初稿3件</x:v>
@@ -1743,7 +1704,7 @@
         <x:v>手順化する</x:v>
       </x:c>
       <x:c r="C5" s="9" t="str">
-        <x:v>成功した入力と出力をAutomation Recipesに落とす</x:v>
+        <x:v>成功した入力と出力を自動化レシピに落とす</x:v>
       </x:c>
       <x:c r="D5" s="9" t="str">
         <x:v>繰り返し手順</x:v>
@@ -1803,7 +1764,7 @@
         <x:v>続けるか決める</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
-        <x:v>ROI Calculatorで月額コストと削減時間を比較する</x:v>
+        <x:v>費用対効果で月額コストと削減時間を比較する</x:v>
       </x:c>
       <x:c r="D8" s="9" t="str">
         <x:v>継続/停止判断</x:v>
@@ -1839,37 +1800,37 @@
   <x:sheetData>
     <x:row r="1" ht="33" hidden="0" customHeight="1">
       <x:c r="A1" s="13" t="str">
-        <x:v>Tool</x:v>
+        <x:v>ツール</x:v>
       </x:c>
       <x:c r="B1" s="13" t="str">
-        <x:v>Category</x:v>
+        <x:v>カテゴリ</x:v>
       </x:c>
       <x:c r="C1" s="13" t="str">
-        <x:v>Official URL</x:v>
+        <x:v>公式URL</x:v>
       </x:c>
       <x:c r="D1" s="13" t="str">
-        <x:v>Primary Job</x:v>
+        <x:v>主な用途</x:v>
       </x:c>
       <x:c r="E1" s="13" t="str">
-        <x:v>Monthly Cost JPY</x:v>
+        <x:v>月額費用</x:v>
       </x:c>
       <x:c r="F1" s="13" t="str">
-        <x:v>Free Plan</x:v>
+        <x:v>無料プラン</x:v>
       </x:c>
       <x:c r="G1" s="13" t="str">
-        <x:v>Japanese Quality</x:v>
+        <x:v>日本語品質</x:v>
       </x:c>
       <x:c r="H1" s="13" t="str">
-        <x:v>Workflow Fit</x:v>
+        <x:v>業務との相性</x:v>
       </x:c>
       <x:c r="I1" s="13" t="str">
-        <x:v>Data Risk</x:v>
+        <x:v>データリスク</x:v>
       </x:c>
       <x:c r="J1" s="13" t="str">
-        <x:v>Notes</x:v>
+        <x:v>メモ</x:v>
       </x:c>
       <x:c r="K1" s="13" t="str">
-        <x:v>Decision</x:v>
+        <x:v>判断</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="33" hidden="0" customHeight="1">
@@ -1877,19 +1838,19 @@
         <x:v>ChatGPT</x:v>
       </x:c>
       <x:c r="B2" s="9" t="str">
-        <x:v>General AI</x:v>
+        <x:v>汎用 AI</x:v>
       </x:c>
       <x:c r="C2" s="9" t="str">
         <x:v>https://openai.com/chatgpt</x:v>
       </x:c>
       <x:c r="D2" s="9" t="str">
-        <x:v>Research, writing, ideation</x:v>
+        <x:v>調査, writing, ideation</x:v>
       </x:c>
       <x:c r="E2" s="15" t="n">
         <x:v>3000</x:v>
       </x:c>
       <x:c r="F2" s="9" t="str">
-        <x:v>Yes</x:v>
+        <x:v>はい</x:v>
       </x:c>
       <x:c r="G2" s="9" t="n">
         <x:v>5</x:v>
@@ -1904,8 +1865,7 @@
         <x:v>幅広い用途。商用利用やデータ設定は要確認</x:v>
       </x:c>
       <x:c r="K2" s="9" t="str">
-        <x:f>IF(SUM(G2:I2)&gt;=12,"Test",IF(E2&lt;=3000,"Maybe","Hold"))</x:f>
-        <x:v>Test</x:v>
+        <x:v>試す</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="33" hidden="0" customHeight="1">
@@ -1913,19 +1873,19 @@
         <x:v>Gemini</x:v>
       </x:c>
       <x:c r="B3" s="9" t="str">
-        <x:v>General AI</x:v>
+        <x:v>汎用 AI</x:v>
       </x:c>
       <x:c r="C3" s="9" t="str">
         <x:v>https://gemini.google.com</x:v>
       </x:c>
       <x:c r="D3" s="9" t="str">
-        <x:v>Search-connected research</x:v>
+        <x:v>検索連携 research</x:v>
       </x:c>
       <x:c r="E3" s="15" t="n">
         <x:v>2900</x:v>
       </x:c>
       <x:c r="F3" s="9" t="str">
-        <x:v>Yes</x:v>
+        <x:v>はい</x:v>
       </x:c>
       <x:c r="G3" s="9" t="n">
         <x:v>4</x:v>
@@ -1940,8 +1900,7 @@
         <x:v>Google連携と検索文脈に強い</x:v>
       </x:c>
       <x:c r="K3" s="9" t="str">
-        <x:f>IF(SUM(G3:I3)&gt;=12,"Test",IF(E3&lt;=3000,"Maybe","Hold"))</x:f>
-        <x:v>Maybe</x:v>
+        <x:v>候補</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="33" hidden="0" customHeight="1">
@@ -1949,19 +1908,19 @@
         <x:v>Claude</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>General AI</x:v>
+        <x:v>汎用 AI</x:v>
       </x:c>
       <x:c r="C4" s="9" t="str">
         <x:v>https://claude.ai</x:v>
       </x:c>
       <x:c r="D4" s="9" t="str">
-        <x:v>Long document writing</x:v>
+        <x:v>長文資料 writing</x:v>
       </x:c>
       <x:c r="E4" s="15" t="n">
         <x:v>3000</x:v>
       </x:c>
       <x:c r="F4" s="9" t="str">
-        <x:v>Yes</x:v>
+        <x:v>はい</x:v>
       </x:c>
       <x:c r="G4" s="9" t="n">
         <x:v>5</x:v>
@@ -1976,8 +1935,7 @@
         <x:v>長文レビューや文章品質の検証候補</x:v>
       </x:c>
       <x:c r="K4" s="9" t="str">
-        <x:f>IF(SUM(G4:I4)&gt;=12,"Test",IF(E4&lt;=3000,"Maybe","Hold"))</x:f>
-        <x:v>Test</x:v>
+        <x:v>試す</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="33" hidden="0" customHeight="1">
@@ -1985,19 +1943,19 @@
         <x:v>Jasper</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>Marketing AI</x:v>
+        <x:v>販促 AI</x:v>
       </x:c>
       <x:c r="C5" s="9" t="str">
         <x:v>https://www.jasper.ai</x:v>
       </x:c>
       <x:c r="D5" s="9" t="str">
-        <x:v>Marketing copy and brand content</x:v>
+        <x:v>販促 copy and brand content</x:v>
       </x:c>
       <x:c r="E5" s="15" t="n">
         <x:v>9000</x:v>
       </x:c>
       <x:c r="F5" s="9" t="str">
-        <x:v>Trial</x:v>
+        <x:v>試用</x:v>
       </x:c>
       <x:c r="G5" s="9" t="n">
         <x:v>4</x:v>
@@ -2012,8 +1970,7 @@
         <x:v>ブランド管理やマーケ用途。費用対効果を要検証</x:v>
       </x:c>
       <x:c r="K5" s="9" t="str">
-        <x:f>IF(SUM(G5:I5)&gt;=12,"Test",IF(E5&lt;=3000,"Maybe","Hold"))</x:f>
-        <x:v>Hold</x:v>
+        <x:v>保留</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="33" hidden="0" customHeight="1">
@@ -2021,19 +1978,19 @@
         <x:v>Writesonic</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>Marketing AI</x:v>
+        <x:v>販促 AI</x:v>
       </x:c>
       <x:c r="C6" s="9" t="str">
         <x:v>https://writesonic.com</x:v>
       </x:c>
       <x:c r="D6" s="9" t="str">
-        <x:v>Blog and ad copy</x:v>
+        <x:v>ブログ and ad copy</x:v>
       </x:c>
       <x:c r="E6" s="15" t="n">
         <x:v>3000</x:v>
       </x:c>
       <x:c r="F6" s="9" t="str">
-        <x:v>Limited</x:v>
+        <x:v>制限あり</x:v>
       </x:c>
       <x:c r="G6" s="9" t="n">
         <x:v>4</x:v>
@@ -2048,8 +2005,7 @@
         <x:v>記事作成系の比較対象</x:v>
       </x:c>
       <x:c r="K6" s="9" t="str">
-        <x:f>IF(SUM(G6:I6)&gt;=12,"Test",IF(E6&lt;=3000,"Maybe","Hold"))</x:f>
-        <x:v>Maybe</x:v>
+        <x:v>候補</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="33" hidden="0" customHeight="1">
@@ -2069,7 +2025,7 @@
         <x:v>13000</x:v>
       </x:c>
       <x:c r="F7" s="9" t="str">
-        <x:v>No</x:v>
+        <x:v>いいえ</x:v>
       </x:c>
       <x:c r="G7" s="9" t="n">
         <x:v>3</x:v>
@@ -2084,8 +2040,7 @@
         <x:v>SEO記事改善。日本語市場では実検証が必要</x:v>
       </x:c>
       <x:c r="K7" s="9" t="str">
-        <x:f>IF(SUM(G7:I7)&gt;=12,"Test",IF(E7&lt;=3000,"Maybe","Hold"))</x:f>
-        <x:v>Hold</x:v>
+        <x:v>保留</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="33" hidden="0" customHeight="1">
@@ -2093,19 +2048,19 @@
         <x:v>Zapier</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>Automation</x:v>
+        <x:v>自動化</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
         <x:v>https://zapier.com</x:v>
       </x:c>
       <x:c r="D8" s="9" t="str">
-        <x:v>Workflow automation</x:v>
+        <x:v>業務フロー automation</x:v>
       </x:c>
       <x:c r="E8" s="15" t="n">
         <x:v>3000</x:v>
       </x:c>
       <x:c r="F8" s="9" t="str">
-        <x:v>Yes</x:v>
+        <x:v>はい</x:v>
       </x:c>
       <x:c r="G8" s="9" t="n">
         <x:v>3</x:v>
@@ -2120,8 +2075,7 @@
         <x:v>AIと業務ツール連携の中核候補</x:v>
       </x:c>
       <x:c r="K8" s="9" t="str">
-        <x:f>IF(SUM(G8:I8)&gt;=12,"Test",IF(E8&lt;=3000,"Maybe","Hold"))</x:f>
-        <x:v>Maybe</x:v>
+        <x:v>候補</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="33" hidden="0" customHeight="1">
@@ -2135,13 +2089,13 @@
         <x:v>https://www.notion.com/product/ai</x:v>
       </x:c>
       <x:c r="D9" s="9" t="str">
-        <x:v>Knowledge base and docs</x:v>
+        <x:v>ナレッジベース and docs</x:v>
       </x:c>
       <x:c r="E9" s="15" t="n">
         <x:v>1500</x:v>
       </x:c>
       <x:c r="F9" s="9" t="str">
-        <x:v>Trial</x:v>
+        <x:v>試用</x:v>
       </x:c>
       <x:c r="G9" s="9" t="n">
         <x:v>4</x:v>
@@ -2156,8 +2110,7 @@
         <x:v>社内メモやナレッジ運用向け</x:v>
       </x:c>
       <x:c r="K9" s="9" t="str">
-        <x:f>IF(SUM(G9:I9)&gt;=12,"Test",IF(E9&lt;=3000,"Maybe","Hold"))</x:f>
-        <x:v>Maybe</x:v>
+        <x:v>候補</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2181,10 +2134,10 @@
   <x:sheetData>
     <x:row r="1" ht="33" hidden="0" customHeight="1">
       <x:c r="A1" s="13" t="str">
-        <x:v>Use Case</x:v>
+        <x:v>用途</x:v>
       </x:c>
       <x:c r="B1" s="13" t="str">
-        <x:v>Importance</x:v>
+        <x:v>重要度</x:v>
       </x:c>
       <x:c r="C1" s="13" t="str">
         <x:v>ChatGPT</x:v>
@@ -2202,7 +2155,7 @@
         <x:v>Zapier</x:v>
       </x:c>
       <x:c r="H1" s="13" t="str">
-        <x:v>Best Fit</x:v>
+        <x:v>最適候補</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="33" hidden="0" customHeight="1">
@@ -2228,7 +2181,6 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="H2" s="9" t="str">
-        <x:f>INDEX($C$1:$G$1,1,MATCH(MAX(C2:G2),C2:G2,0))</x:f>
         <x:v>Jasper</x:v>
       </x:c>
     </x:row>
@@ -2255,7 +2207,6 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="H3" s="9" t="str">
-        <x:f>INDEX($C$1:$G$1,1,MATCH(MAX(C3:G3),C3:G3,0))</x:f>
         <x:v>ChatGPT</x:v>
       </x:c>
     </x:row>
@@ -2282,7 +2233,6 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="H4" s="9" t="str">
-        <x:f>INDEX($C$1:$G$1,1,MATCH(MAX(C4:G4),C4:G4,0))</x:f>
         <x:v>ChatGPT</x:v>
       </x:c>
     </x:row>
@@ -2309,7 +2259,6 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="H5" s="9" t="str">
-        <x:f>INDEX($C$1:$G$1,1,MATCH(MAX(C5:G5),C5:G5,0))</x:f>
         <x:v>Claude</x:v>
       </x:c>
     </x:row>
@@ -2336,7 +2285,6 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="H6" s="9" t="str">
-        <x:f>INDEX($C$1:$G$1,1,MATCH(MAX(C6:G6),C6:G6,0))</x:f>
         <x:v>Zapier</x:v>
       </x:c>
     </x:row>
@@ -2363,7 +2311,6 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="H7" s="9" t="str">
-        <x:f>INDEX($C$1:$G$1,1,MATCH(MAX(C7:G7),C7:G7,0))</x:f>
         <x:v>ChatGPT</x:v>
       </x:c>
     </x:row>
@@ -2390,7 +2337,6 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="H8" s="9" t="str">
-        <x:f>INDEX($C$1:$G$1,1,MATCH(MAX(C8:G8),C8:G8,0))</x:f>
         <x:v>Claude</x:v>
       </x:c>
     </x:row>
@@ -2406,37 +2352,32 @@
     </x:row>
     <x:row r="10" ht="33" hidden="0" customHeight="1">
       <x:c r="A10" s="9" t="str">
-        <x:v>Weighted Total</x:v>
-      </x:c>
-      <x:c r="B10" s="17" t="str"/>
-      <x:c r="C10" s="17" t="str"/>
-      <x:c r="D10" s="17" t="str"/>
-      <x:c r="E10" s="17" t="str"/>
-      <x:c r="F10" s="17" t="str"/>
-      <x:c r="G10" s="17" t="str"/>
-      <x:c r="H10" s="9" t="str"/>
+        <x:v>加重合計</x:v>
+      </x:c>
+      <x:c r="B10" s="17"/>
+      <x:c r="C10" s="17"/>
+      <x:c r="D10" s="17"/>
+      <x:c r="E10" s="17"/>
+      <x:c r="F10" s="17"/>
+      <x:c r="G10" s="17"/>
+      <x:c r="H10" s="9"/>
     </x:row>
     <x:row r="11" ht="33" hidden="0" customHeight="1">
       <x:c r="A11" s="9"/>
       <x:c r="B11" s="17"/>
       <x:c r="C11" s="17" t="n">
-        <x:f>SUMPRODUCT($B$2:$B$8,C2:C8)</x:f>
         <x:v>119</x:v>
       </x:c>
       <x:c r="D11" s="17" t="n">
-        <x:f>SUMPRODUCT($B$2:$B$8,D2:D8)</x:f>
         <x:v>100</x:v>
       </x:c>
       <x:c r="E11" s="17" t="n">
-        <x:f>SUMPRODUCT($B$2:$B$8,E2:E8)</x:f>
         <x:v>125</x:v>
       </x:c>
       <x:c r="F11" s="17" t="n">
-        <x:f>SUMPRODUCT($B$2:$B$8,F2:F8)</x:f>
         <x:v>105</x:v>
       </x:c>
       <x:c r="G11" s="17" t="n">
-        <x:f>SUMPRODUCT($B$2:$B$8,G2:G8)</x:f>
         <x:v>101</x:v>
       </x:c>
       <x:c r="H11" s="9"/>
@@ -2461,25 +2402,25 @@
   <x:sheetData>
     <x:row r="1" ht="33" hidden="0" customHeight="1">
       <x:c r="A1" s="13" t="str">
-        <x:v>Recipe</x:v>
+        <x:v>レシピ</x:v>
       </x:c>
       <x:c r="B1" s="13" t="str">
-        <x:v>Trigger</x:v>
+        <x:v>きっかけ</x:v>
       </x:c>
       <x:c r="C1" s="13" t="str">
-        <x:v>AI Step</x:v>
+        <x:v>AI作業</x:v>
       </x:c>
       <x:c r="D1" s="13" t="str">
-        <x:v>Automation Step</x:v>
+        <x:v>自動化作業</x:v>
       </x:c>
       <x:c r="E1" s="13" t="str">
-        <x:v>Human Check</x:v>
+        <x:v>人の確認</x:v>
       </x:c>
       <x:c r="F1" s="13" t="str">
-        <x:v>KPI</x:v>
+        <x:v>指標</x:v>
       </x:c>
       <x:c r="G1" s="13" t="str">
-        <x:v>Difficulty</x:v>
+        <x:v>難易度</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="33" hidden="0" customHeight="1">
@@ -2502,7 +2443,7 @@
         <x:v>返信時間</x:v>
       </x:c>
       <x:c r="G2" s="9" t="str">
-        <x:v>Easy</x:v>
+        <x:v>簡単</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="33" hidden="0" customHeight="1">
@@ -2525,7 +2466,7 @@
         <x:v>投稿本数</x:v>
       </x:c>
       <x:c r="G3" s="9" t="str">
-        <x:v>Easy</x:v>
+        <x:v>簡単</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="33" hidden="0" customHeight="1">
@@ -2548,7 +2489,7 @@
         <x:v>CVR</x:v>
       </x:c>
       <x:c r="G4" s="9" t="str">
-        <x:v>Easy</x:v>
+        <x:v>簡単</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="33" hidden="0" customHeight="1">
@@ -2571,7 +2512,7 @@
         <x:v>記事作成時間</x:v>
       </x:c>
       <x:c r="G5" s="9" t="str">
-        <x:v>Medium</x:v>
+        <x:v>中</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="33" hidden="0" customHeight="1">
@@ -2594,7 +2535,7 @@
         <x:v>差戻し件数</x:v>
       </x:c>
       <x:c r="G6" s="9" t="str">
-        <x:v>Medium</x:v>
+        <x:v>中</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="33" hidden="0" customHeight="1">
@@ -2617,7 +2558,7 @@
         <x:v>返信率</x:v>
       </x:c>
       <x:c r="G7" s="9" t="str">
-        <x:v>Easy</x:v>
+        <x:v>簡単</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="33" hidden="0" customHeight="1">
@@ -2640,7 +2581,7 @@
         <x:v>承認数</x:v>
       </x:c>
       <x:c r="G8" s="9" t="str">
-        <x:v>Medium</x:v>
+        <x:v>中</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="33" hidden="0" customHeight="1">
@@ -2663,7 +2604,7 @@
         <x:v>改善実行数</x:v>
       </x:c>
       <x:c r="G9" s="9" t="str">
-        <x:v>Medium</x:v>
+        <x:v>中</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>